<commit_message>
Preparations for forces and loads calculation
Concretise sizes and lengthies
Recalculated and updated shafts keys
Updated case sizes and model
</commit_message>
<xml_diff>
--- a/Расчёт.xlsx
+++ b/Расчёт.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Professional\Downloads\интститут\курсач детмаш\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B752255A-80C5-48CC-B3F0-B1CFEA11A6BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A73725F4-E076-4A54-ABF6-ACEC85FEB3A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="812" activeTab="1" xr2:uid="{7E097F76-7D13-4899-AD2E-10ADA644057F}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="812" activeTab="8" xr2:uid="{7E097F76-7D13-4899-AD2E-10ADA644057F}"/>
   </bookViews>
   <sheets>
     <sheet name="Электродвигатель" sheetId="1" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="769" uniqueCount="378">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="801" uniqueCount="382">
   <si>
     <t>Окружная сила</t>
   </si>
@@ -1162,9 +1162,6 @@
     <t>Ширина b</t>
   </si>
   <si>
-    <t>Шпонка</t>
-  </si>
-  <si>
     <t>Высота шпонки h</t>
   </si>
   <si>
@@ -1174,13 +1171,28 @@
     <t>Глубина паза t1 (вала)</t>
   </si>
   <si>
-    <t>Материал вала</t>
-  </si>
-  <si>
     <t>Предел текучести</t>
   </si>
   <si>
     <t>Предел на смятие</t>
+  </si>
+  <si>
+    <t>Предел на смятие шпонки</t>
+  </si>
+  <si>
+    <t>Расчёт длинны шпонки из условия несмятия</t>
+  </si>
+  <si>
+    <t>МПа</t>
+  </si>
+  <si>
+    <t>Рабочая длинна шпонки</t>
+  </si>
+  <si>
+    <t>Минимальная высота шпонки</t>
+  </si>
+  <si>
+    <t>Высота смятия шпонки</t>
   </si>
 </sst>
 </file>
@@ -2053,16 +2065,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>510540</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>45720</xdr:rowOff>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>182880</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>167640</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>501865</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>44096</xdr:rowOff>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>174205</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>166016</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2085,7 +2097,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4168140" y="960120"/>
+          <a:off x="7299960" y="167640"/>
           <a:ext cx="6087325" cy="2010056"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -10360,6 +10372,9 @@
     <mergeCell ref="J14:L14"/>
     <mergeCell ref="Z6:AA6"/>
     <mergeCell ref="Z11:AA11"/>
+    <mergeCell ref="Z10:AA10"/>
+    <mergeCell ref="X10:Y10"/>
+    <mergeCell ref="J13:L13"/>
     <mergeCell ref="Z3:AA3"/>
     <mergeCell ref="T3:W3"/>
     <mergeCell ref="T4:W4"/>
@@ -10367,10 +10382,7 @@
     <mergeCell ref="X4:Y4"/>
     <mergeCell ref="X5:Y5"/>
     <mergeCell ref="X3:Y3"/>
-    <mergeCell ref="Z10:AA10"/>
-    <mergeCell ref="X10:Y10"/>
     <mergeCell ref="Z5:AA5"/>
-    <mergeCell ref="J13:L13"/>
     <mergeCell ref="J11:L11"/>
     <mergeCell ref="J12:L12"/>
     <mergeCell ref="X11:Y11"/>
@@ -10447,7 +10459,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F31C697-F4FB-4FAD-9F40-0B2C485D61BE}">
-  <dimension ref="A2:F37"/>
+  <dimension ref="A2:G43"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="20" width="6.77734375" customWidth="1"/>
@@ -10557,7 +10569,7 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="124" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="B10" s="124"/>
       <c r="C10" s="124"/>
@@ -10569,7 +10581,7 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="124" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="B11" s="124"/>
       <c r="C11" s="124"/>
@@ -10643,8 +10655,8 @@
       <c r="C30" s="124"/>
       <c r="D30" s="124"/>
       <c r="E30">
-        <f>Вал!$K$13</f>
-        <v>32</v>
+        <f ca="1">Вал!S12</f>
+        <v>40</v>
       </c>
       <c r="F30" t="s">
         <v>16</v>
@@ -10652,12 +10664,13 @@
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" s="124" t="s">
-        <v>371</v>
+        <v>377</v>
       </c>
       <c r="B31" s="124"/>
       <c r="C31" s="124"/>
       <c r="D31" s="124"/>
       <c r="E31" s="124"/>
+      <c r="F31" s="124"/>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" s="124" t="s">
@@ -10667,15 +10680,15 @@
       <c r="C32" s="124"/>
       <c r="D32" s="124"/>
       <c r="E32" s="52">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F32" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A33" s="124" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="B33" s="124"/>
       <c r="C33" s="124"/>
@@ -10687,9 +10700,9 @@
         <v>16</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A34" s="124" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="B34" s="124"/>
       <c r="C34" s="124"/>
@@ -10701,7 +10714,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35" s="124" t="s">
         <v>206</v>
       </c>
@@ -10715,9 +10728,9 @@
         <v>16</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A36" s="124" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="B36" s="124"/>
       <c r="C36" s="124"/>
@@ -10729,16 +10742,93 @@
         <v>16</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A37" s="124" t="s">
-        <v>375</v>
-      </c>
-      <c r="B37" s="124"/>
-      <c r="C37" s="124"/>
-      <c r="D37" s="124"/>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A37" s="48"/>
+      <c r="B37" s="48"/>
+      <c r="C37" s="48"/>
+      <c r="D37" s="48"/>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A38" s="124" t="s">
+        <v>381</v>
+      </c>
+      <c r="B38" s="124"/>
+      <c r="C38" s="124"/>
+      <c r="D38" s="124"/>
+      <c r="E38">
+        <f>MIN(E34,E33-E34)</f>
+        <v>3</v>
+      </c>
+      <c r="F38" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A39" s="124" t="s">
+        <v>376</v>
+      </c>
+      <c r="B39" s="124"/>
+      <c r="C39" s="124"/>
+      <c r="D39" s="124"/>
+      <c r="E39" s="52">
+        <v>110</v>
+      </c>
+      <c r="F39" t="s">
+        <v>378</v>
+      </c>
+      <c r="G39" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A40" s="124" t="s">
+        <v>379</v>
+      </c>
+      <c r="B40" s="124"/>
+      <c r="C40" s="124"/>
+      <c r="D40" s="124"/>
+      <c r="E40">
+        <f ca="1">E29*2*1000/E30/E39/E38</f>
+        <v>51.939287331535837</v>
+      </c>
+      <c r="F40" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A41" s="124" t="s">
+        <v>201</v>
+      </c>
+      <c r="B41" s="124"/>
+      <c r="C41" s="124"/>
+      <c r="D41" s="124"/>
+      <c r="E41">
+        <f ca="1">E40+E32</f>
+        <v>63.939287331535837</v>
+      </c>
+      <c r="F41" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A42" s="48"/>
+      <c r="B42" s="48"/>
+      <c r="C42" s="48"/>
+      <c r="D42" s="48"/>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A43" s="48"/>
+      <c r="B43" s="48"/>
+      <c r="C43" s="48"/>
+      <c r="D43" s="48"/>
     </row>
   </sheetData>
-  <mergeCells count="23">
+  <mergeCells count="26">
+    <mergeCell ref="A31:F31"/>
+    <mergeCell ref="A41:D41"/>
+    <mergeCell ref="A38:D38"/>
+    <mergeCell ref="A39:D39"/>
+    <mergeCell ref="A40:D40"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="A24:D24"/>
     <mergeCell ref="A25:D25"/>
@@ -10752,14 +10842,12 @@
     <mergeCell ref="A6:D6"/>
     <mergeCell ref="A35:D35"/>
     <mergeCell ref="A36:D36"/>
-    <mergeCell ref="A37:D37"/>
     <mergeCell ref="A9:D9"/>
     <mergeCell ref="A10:D10"/>
     <mergeCell ref="A11:D11"/>
     <mergeCell ref="A29:D29"/>
     <mergeCell ref="A30:D30"/>
     <mergeCell ref="A32:D32"/>
-    <mergeCell ref="A31:E31"/>
     <mergeCell ref="A34:D34"/>
     <mergeCell ref="A33:D33"/>
   </mergeCells>
@@ -10770,9 +10858,212 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4CC16526-A479-4083-A8A6-C1DA4D6AD8E8}">
-  <dimension ref="A1"/>
+  <dimension ref="A6:F19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="14" width="6.77734375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" s="124" t="s">
+        <v>369</v>
+      </c>
+      <c r="B6" s="124"/>
+      <c r="C6" s="124"/>
+      <c r="D6" s="124"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" s="124" t="s">
+        <v>166</v>
+      </c>
+      <c r="B7" s="124"/>
+      <c r="C7" s="124"/>
+      <c r="D7" s="124"/>
+      <c r="E7" s="61">
+        <f>Электродвигатель!$P$53</f>
+        <v>48.741201321892952</v>
+      </c>
+      <c r="F7" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8" s="124" t="s">
+        <v>118</v>
+      </c>
+      <c r="B8" s="124"/>
+      <c r="C8" s="124"/>
+      <c r="D8" s="124"/>
+      <c r="E8">
+        <f>Вал!K13</f>
+        <v>32</v>
+      </c>
+      <c r="F8" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9" s="124" t="s">
+        <v>377</v>
+      </c>
+      <c r="B9" s="124"/>
+      <c r="C9" s="124"/>
+      <c r="D9" s="124"/>
+      <c r="E9" s="124"/>
+      <c r="F9" s="124"/>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10" s="124" t="s">
+        <v>370</v>
+      </c>
+      <c r="B10" s="124"/>
+      <c r="C10" s="124"/>
+      <c r="D10" s="124"/>
+      <c r="E10" s="52">
+        <v>10</v>
+      </c>
+      <c r="F10" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11" s="124" t="s">
+        <v>371</v>
+      </c>
+      <c r="B11" s="124"/>
+      <c r="C11" s="124"/>
+      <c r="D11" s="124"/>
+      <c r="E11" s="52">
+        <v>8</v>
+      </c>
+      <c r="F11" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A12" s="124" t="s">
+        <v>373</v>
+      </c>
+      <c r="B12" s="124"/>
+      <c r="C12" s="124"/>
+      <c r="D12" s="124"/>
+      <c r="E12" s="52">
+        <v>5</v>
+      </c>
+      <c r="F12" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A13" s="124" t="s">
+        <v>206</v>
+      </c>
+      <c r="B13" s="124"/>
+      <c r="C13" s="124"/>
+      <c r="D13" s="124"/>
+      <c r="E13" s="52">
+        <v>0.5</v>
+      </c>
+      <c r="F13" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14" s="124" t="s">
+        <v>372</v>
+      </c>
+      <c r="B14" s="124"/>
+      <c r="C14" s="124"/>
+      <c r="D14" s="124"/>
+      <c r="E14" s="52">
+        <v>3.3</v>
+      </c>
+      <c r="F14" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A15" s="48"/>
+      <c r="B15" s="48"/>
+      <c r="C15" s="48"/>
+      <c r="D15" s="48"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A16" s="124" t="s">
+        <v>380</v>
+      </c>
+      <c r="B16" s="124"/>
+      <c r="C16" s="124"/>
+      <c r="D16" s="124"/>
+      <c r="E16">
+        <f>MIN(E12,E11-E12)</f>
+        <v>3</v>
+      </c>
+      <c r="F16" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A17" s="124" t="s">
+        <v>376</v>
+      </c>
+      <c r="B17" s="124"/>
+      <c r="C17" s="124"/>
+      <c r="D17" s="124"/>
+      <c r="E17" s="90">
+        <f>'тихоходный вал'!E39</f>
+        <v>110</v>
+      </c>
+      <c r="F17" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A18" s="124" t="s">
+        <v>379</v>
+      </c>
+      <c r="B18" s="124"/>
+      <c r="C18" s="124"/>
+      <c r="D18" s="124"/>
+      <c r="E18">
+        <f>E7*2*1000/E8/E17/E16</f>
+        <v>9.2312881291463924</v>
+      </c>
+      <c r="F18" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A19" s="124" t="s">
+        <v>201</v>
+      </c>
+      <c r="B19" s="124"/>
+      <c r="C19" s="124"/>
+      <c r="D19" s="124"/>
+      <c r="E19">
+        <f>E18+E10</f>
+        <v>19.231288129146392</v>
+      </c>
+      <c r="F19" t="s">
+        <v>16</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="13">
+    <mergeCell ref="A16:D16"/>
+    <mergeCell ref="A17:D17"/>
+    <mergeCell ref="A18:D18"/>
+    <mergeCell ref="A19:D19"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="A7:D7"/>
+    <mergeCell ref="A8:D8"/>
+    <mergeCell ref="A9:F9"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="A11:D11"/>
+    <mergeCell ref="A12:D12"/>
+    <mergeCell ref="A13:D13"/>
+    <mergeCell ref="A14:D14"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Started force and load calculation
</commit_message>
<xml_diff>
--- a/Расчёт.xlsx
+++ b/Расчёт.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Professional\Downloads\интститут\курсач детмаш\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A73725F4-E076-4A54-ABF6-ACEC85FEB3A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{966D5585-7C20-4BA9-AA75-12DC92CCF878}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="812" activeTab="8" xr2:uid="{7E097F76-7D13-4899-AD2E-10ADA644057F}"/>
   </bookViews>
@@ -20,10 +20,11 @@
     <sheet name="Колесо" sheetId="7" r:id="rId5"/>
     <sheet name="тихоходный вал" sheetId="14" r:id="rId6"/>
     <sheet name="вал-шестерня" sheetId="13" r:id="rId7"/>
-    <sheet name="Корпус" sheetId="3" r:id="rId8"/>
-    <sheet name="Ra40" sheetId="5" r:id="rId9"/>
-    <sheet name="Подшипники" sheetId="10" r:id="rId10"/>
-    <sheet name="Материалы" sheetId="11" r:id="rId11"/>
+    <sheet name="силы" sheetId="15" r:id="rId8"/>
+    <sheet name="Корпус" sheetId="3" r:id="rId9"/>
+    <sheet name="Ra40" sheetId="5" r:id="rId10"/>
+    <sheet name="Подшипники" sheetId="10" r:id="rId11"/>
+    <sheet name="Материалы" sheetId="11" r:id="rId12"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -47,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="801" uniqueCount="382">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="842" uniqueCount="393">
   <si>
     <t>Окружная сила</t>
   </si>
@@ -1193,6 +1194,39 @@
   </si>
   <si>
     <t>Высота смятия шпонки</t>
+  </si>
+  <si>
+    <t>Расчёт сил в узлах</t>
+  </si>
+  <si>
+    <t>Длинны</t>
+  </si>
+  <si>
+    <t>Длинна 12</t>
+  </si>
+  <si>
+    <t>Длинна 23</t>
+  </si>
+  <si>
+    <t>Длинна 34</t>
+  </si>
+  <si>
+    <t>Радиальная косольная сила</t>
+  </si>
+  <si>
+    <t>Осевая сила Fa</t>
+  </si>
+  <si>
+    <t>Радиальная сила Fr</t>
+  </si>
+  <si>
+    <t>Окружная сила Ft</t>
+  </si>
+  <si>
+    <t>Окружная консольная сила</t>
+  </si>
+  <si>
+    <t>Эквиавлетные коэффициент нагружения</t>
   </si>
 </sst>
 </file>
@@ -4328,10 +4362,10 @@
         <v>0.77619649168341942</v>
       </c>
       <c r="AB42">
-        <v>183</v>
+        <v>177</v>
       </c>
       <c r="AC42" t="s">
-        <v>309</v>
+        <v>382</v>
       </c>
     </row>
     <row r="43" spans="2:29" x14ac:dyDescent="0.3">
@@ -4409,9 +4443,6 @@
         <f t="shared" ca="1" si="16"/>
         <v>0.77322226173177433</v>
       </c>
-      <c r="AC43" t="s">
-        <v>310</v>
-      </c>
     </row>
     <row r="44" spans="2:29" x14ac:dyDescent="0.3">
       <c r="C44" s="1"/>
@@ -4482,8 +4513,11 @@
         <f t="shared" ca="1" si="16"/>
         <v>0</v>
       </c>
-      <c r="AC44" s="1" t="s">
-        <v>311</v>
+      <c r="AB44">
+        <v>183</v>
+      </c>
+      <c r="AC44" t="s">
+        <v>309</v>
       </c>
     </row>
     <row r="45" spans="2:29" x14ac:dyDescent="0.3">
@@ -4552,8 +4586,8 @@
         <f t="shared" ca="1" si="16"/>
         <v>0</v>
       </c>
-      <c r="AC45" s="1" t="s">
-        <v>312</v>
+      <c r="AC45" t="s">
+        <v>310</v>
       </c>
     </row>
     <row r="46" spans="2:29" x14ac:dyDescent="0.3">
@@ -4632,6 +4666,9 @@
       <c r="Z46" s="5">
         <f t="shared" ca="1" si="16"/>
         <v>0.75835111197354876</v>
+      </c>
+      <c r="AC46" s="1" t="s">
+        <v>311</v>
       </c>
     </row>
     <row r="47" spans="2:29" x14ac:dyDescent="0.3">
@@ -4660,8 +4697,8 @@
       <c r="X47" s="1"/>
       <c r="Y47" s="30"/>
       <c r="Z47" s="1"/>
-      <c r="AC47" s="25" t="s">
-        <v>320</v>
+      <c r="AC47" s="1" t="s">
+        <v>312</v>
       </c>
     </row>
     <row r="48" spans="2:29" x14ac:dyDescent="0.3">
@@ -4699,9 +4736,6 @@
       <c r="X48" s="1"/>
       <c r="Y48" s="30"/>
       <c r="Z48" s="1"/>
-      <c r="AC48" s="25" t="s">
-        <v>313</v>
-      </c>
     </row>
     <row r="49" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B49" s="99" t="s">
@@ -4732,6 +4766,9 @@
       <c r="X49" s="1"/>
       <c r="Y49" s="30"/>
       <c r="Z49" s="1"/>
+      <c r="AC49" s="25" t="s">
+        <v>320</v>
+      </c>
     </row>
     <row r="50" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B50" s="99" t="s">
@@ -4754,8 +4791,8 @@
       <c r="X50" s="1"/>
       <c r="Y50" s="30"/>
       <c r="Z50" s="1"/>
-      <c r="AC50" s="1" t="s">
-        <v>321</v>
+      <c r="AC50" s="25" t="s">
+        <v>313</v>
       </c>
     </row>
     <row r="51" spans="2:29" x14ac:dyDescent="0.3">
@@ -4802,9 +4839,6 @@
       <c r="X51" s="1"/>
       <c r="Y51" s="30"/>
       <c r="Z51" s="1"/>
-      <c r="AC51" s="49" t="s">
-        <v>307</v>
-      </c>
     </row>
     <row r="52" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B52" s="99" t="s">
@@ -4853,6 +4887,9 @@
       <c r="X52" s="1"/>
       <c r="Y52" s="30"/>
       <c r="Z52" s="1"/>
+      <c r="AC52" s="1" t="s">
+        <v>321</v>
+      </c>
     </row>
     <row r="53" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B53" s="99" t="s">
@@ -4902,6 +4939,9 @@
       <c r="X53" s="36"/>
       <c r="Y53" s="30"/>
       <c r="Z53" s="1"/>
+      <c r="AC53" s="49" t="s">
+        <v>307</v>
+      </c>
     </row>
     <row r="54" spans="2:29" x14ac:dyDescent="0.3">
       <c r="B54" s="99" t="s">
@@ -5344,6 +5384,659 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D8564D3-007A-4908-B584-B11BCC9DA655}">
+  <dimension ref="A1:E80"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" s="124">
+        <v>1</v>
+      </c>
+      <c r="B1">
+        <v>1</v>
+      </c>
+      <c r="D1" s="48"/>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" s="124"/>
+      <c r="B2">
+        <v>1.05</v>
+      </c>
+      <c r="D2" s="48"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" s="124">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B3">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="D3" s="48"/>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" s="124"/>
+      <c r="B4">
+        <v>1.1499999999999999</v>
+      </c>
+      <c r="D4" s="48"/>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" s="124">
+        <v>1.2</v>
+      </c>
+      <c r="B5">
+        <v>1.2</v>
+      </c>
+      <c r="D5" s="48"/>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" s="124"/>
+      <c r="B6">
+        <v>1.3</v>
+      </c>
+      <c r="D6" s="48"/>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" s="124">
+        <v>1.4</v>
+      </c>
+      <c r="B7">
+        <v>1.4</v>
+      </c>
+      <c r="D7" s="48"/>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" s="124"/>
+      <c r="B8">
+        <v>1.5</v>
+      </c>
+      <c r="D8" s="48"/>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" s="124">
+        <v>1.6</v>
+      </c>
+      <c r="B9">
+        <v>1.6</v>
+      </c>
+      <c r="D9" s="48"/>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A10" s="124"/>
+      <c r="B10">
+        <v>1.7</v>
+      </c>
+      <c r="D10" s="48"/>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A11" s="124">
+        <v>1.8</v>
+      </c>
+      <c r="B11">
+        <v>1.8</v>
+      </c>
+      <c r="D11" s="48"/>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A12" s="124"/>
+      <c r="B12">
+        <v>1.9</v>
+      </c>
+      <c r="D12" s="48"/>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A13" s="124">
+        <v>2</v>
+      </c>
+      <c r="B13">
+        <v>2</v>
+      </c>
+      <c r="D13" s="48"/>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A14" s="124"/>
+      <c r="B14">
+        <v>2.1</v>
+      </c>
+      <c r="D14" s="48"/>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A15" s="124">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B15">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="D15" s="48"/>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A16" s="124"/>
+      <c r="B16">
+        <v>2.4</v>
+      </c>
+      <c r="D16" s="48"/>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A17" s="124">
+        <v>2.5</v>
+      </c>
+      <c r="B17">
+        <v>2.5</v>
+      </c>
+      <c r="D17" s="48"/>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A18" s="124"/>
+      <c r="B18">
+        <v>2.6</v>
+      </c>
+      <c r="D18" s="48"/>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A19" s="124">
+        <v>2.8</v>
+      </c>
+      <c r="B19">
+        <v>2.8</v>
+      </c>
+      <c r="D19" s="48"/>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A20" s="124"/>
+      <c r="B20">
+        <v>3</v>
+      </c>
+      <c r="D20" s="48"/>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A21" s="124">
+        <v>3.2</v>
+      </c>
+      <c r="B21">
+        <v>3.2</v>
+      </c>
+      <c r="D21" s="48"/>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A22" s="124"/>
+      <c r="B22">
+        <v>3.4</v>
+      </c>
+      <c r="D22" s="48"/>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A23" s="124">
+        <v>3.6</v>
+      </c>
+      <c r="B23">
+        <v>3.6</v>
+      </c>
+      <c r="D23" s="48"/>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A24" s="124"/>
+      <c r="B24">
+        <v>3.8</v>
+      </c>
+      <c r="D24" s="48"/>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A25" s="124">
+        <v>4</v>
+      </c>
+      <c r="B25">
+        <v>4</v>
+      </c>
+      <c r="D25" s="48"/>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A26" s="124"/>
+      <c r="B26">
+        <v>4.2</v>
+      </c>
+      <c r="D26" s="48"/>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A27" s="124">
+        <v>4.5</v>
+      </c>
+      <c r="B27">
+        <v>4.5</v>
+      </c>
+      <c r="D27" s="48"/>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A28" s="124"/>
+      <c r="B28">
+        <v>4.8</v>
+      </c>
+      <c r="D28" s="48"/>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A29" s="124">
+        <v>5</v>
+      </c>
+      <c r="B29">
+        <v>5</v>
+      </c>
+      <c r="D29" s="48"/>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A30" s="124"/>
+      <c r="B30">
+        <v>5.3</v>
+      </c>
+      <c r="D30" s="48"/>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A31" s="124">
+        <v>5.6</v>
+      </c>
+      <c r="B31">
+        <v>5.6</v>
+      </c>
+      <c r="D31" s="48"/>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A32" s="124"/>
+      <c r="B32">
+        <v>6</v>
+      </c>
+      <c r="D32" s="48"/>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A33" s="124">
+        <v>6.3</v>
+      </c>
+      <c r="B33">
+        <v>6.3</v>
+      </c>
+      <c r="D33" s="48"/>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A34" s="124"/>
+      <c r="B34">
+        <v>6.7</v>
+      </c>
+      <c r="D34" s="48"/>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A35" s="124">
+        <v>7.1</v>
+      </c>
+      <c r="B35">
+        <v>7.1</v>
+      </c>
+      <c r="D35" s="48"/>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A36" s="124"/>
+      <c r="B36">
+        <v>7.5</v>
+      </c>
+      <c r="D36" s="48"/>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A37" s="124">
+        <v>8</v>
+      </c>
+      <c r="B37">
+        <v>8</v>
+      </c>
+      <c r="D37" s="48"/>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A38" s="124"/>
+      <c r="B38">
+        <v>8.5</v>
+      </c>
+      <c r="D38" s="48"/>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A39" s="124">
+        <v>9</v>
+      </c>
+      <c r="B39">
+        <v>9</v>
+      </c>
+      <c r="D39" s="48"/>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A40" s="124"/>
+      <c r="B40" s="61">
+        <v>9.5</v>
+      </c>
+      <c r="D40" s="48"/>
+      <c r="E40" s="61"/>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A41" s="124">
+        <v>10</v>
+      </c>
+      <c r="B41" s="48">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A42" s="124"/>
+      <c r="B42" s="48">
+        <v>10.5</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A43" s="124">
+        <v>11</v>
+      </c>
+      <c r="B43" s="48">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A44" s="124"/>
+      <c r="B44" s="48">
+        <v>11.5</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A45" s="124">
+        <v>12</v>
+      </c>
+      <c r="B45" s="48">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A46" s="124"/>
+      <c r="B46" s="48">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A47" s="124">
+        <v>14</v>
+      </c>
+      <c r="B47" s="48">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A48" s="124"/>
+      <c r="B48" s="48">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A49" s="124">
+        <v>16</v>
+      </c>
+      <c r="B49" s="48">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A50" s="124"/>
+      <c r="B50" s="48">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A51" s="124">
+        <v>18</v>
+      </c>
+      <c r="B51" s="48">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A52" s="124"/>
+      <c r="B52" s="48">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A53" s="124">
+        <v>20</v>
+      </c>
+      <c r="B53" s="48">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A54" s="124"/>
+      <c r="B54" s="48">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A55" s="124">
+        <v>22</v>
+      </c>
+      <c r="B55" s="48">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A56" s="124"/>
+      <c r="B56" s="48">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A57" s="124">
+        <v>25</v>
+      </c>
+      <c r="B57" s="48">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A58" s="124"/>
+      <c r="B58" s="48">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A59" s="124">
+        <v>28</v>
+      </c>
+      <c r="B59" s="48">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A60" s="124"/>
+      <c r="B60" s="48">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A61" s="124">
+        <v>32</v>
+      </c>
+      <c r="B61" s="48">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A62" s="124"/>
+      <c r="B62" s="48">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A63" s="124">
+        <v>36</v>
+      </c>
+      <c r="B63" s="48">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A64" s="124"/>
+      <c r="B64" s="48">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A65" s="124">
+        <v>40</v>
+      </c>
+      <c r="B65" s="48">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A66" s="124"/>
+      <c r="B66" s="48">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A67" s="124">
+        <v>45</v>
+      </c>
+      <c r="B67" s="48">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A68" s="124"/>
+      <c r="B68" s="48">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A69" s="124">
+        <v>50</v>
+      </c>
+      <c r="B69" s="48">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A70" s="124"/>
+      <c r="B70" s="48">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A71" s="124">
+        <v>56</v>
+      </c>
+      <c r="B71" s="48">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A72" s="124"/>
+      <c r="B72" s="48">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A73" s="124">
+        <v>63</v>
+      </c>
+      <c r="B73" s="48">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A74" s="124"/>
+      <c r="B74" s="48">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A75" s="124">
+        <v>71</v>
+      </c>
+      <c r="B75" s="48">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A76" s="124"/>
+      <c r="B76" s="48">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A77" s="124">
+        <v>80</v>
+      </c>
+      <c r="B77" s="48">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A78" s="124"/>
+      <c r="B78" s="48">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A79" s="124">
+        <v>90</v>
+      </c>
+      <c r="B79" s="48">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A80" s="124"/>
+      <c r="B80" s="48">
+        <v>95</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="40">
+    <mergeCell ref="A77:A78"/>
+    <mergeCell ref="A79:A80"/>
+    <mergeCell ref="A65:A66"/>
+    <mergeCell ref="A67:A68"/>
+    <mergeCell ref="A69:A70"/>
+    <mergeCell ref="A71:A72"/>
+    <mergeCell ref="A73:A74"/>
+    <mergeCell ref="A75:A76"/>
+    <mergeCell ref="A63:A64"/>
+    <mergeCell ref="A41:A42"/>
+    <mergeCell ref="A43:A44"/>
+    <mergeCell ref="A45:A46"/>
+    <mergeCell ref="A47:A48"/>
+    <mergeCell ref="A49:A50"/>
+    <mergeCell ref="A51:A52"/>
+    <mergeCell ref="A53:A54"/>
+    <mergeCell ref="A55:A56"/>
+    <mergeCell ref="A57:A58"/>
+    <mergeCell ref="A59:A60"/>
+    <mergeCell ref="A61:A62"/>
+    <mergeCell ref="A37:A38"/>
+    <mergeCell ref="A39:A40"/>
+    <mergeCell ref="A25:A26"/>
+    <mergeCell ref="A27:A28"/>
+    <mergeCell ref="A29:A30"/>
+    <mergeCell ref="A31:A32"/>
+    <mergeCell ref="A33:A34"/>
+    <mergeCell ref="A35:A36"/>
+    <mergeCell ref="A23:A24"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="A3:A4"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="A7:A8"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="A13:A14"/>
+    <mergeCell ref="A15:A16"/>
+    <mergeCell ref="A17:A18"/>
+    <mergeCell ref="A19:A20"/>
+    <mergeCell ref="A21:A22"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D136A9F2-8845-4295-A8BD-25F04BE0EFA0}">
   <dimension ref="A1:T34"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -6058,7 +6751,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32704C68-B145-4DB6-B0E3-AE1BF65D15BC}">
   <dimension ref="A1:L14"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -10771,7 +11464,7 @@
       <c r="C39" s="124"/>
       <c r="D39" s="124"/>
       <c r="E39" s="52">
-        <v>110</v>
+        <v>120</v>
       </c>
       <c r="F39" t="s">
         <v>378</v>
@@ -10789,7 +11482,7 @@
       <c r="D40" s="124"/>
       <c r="E40">
         <f ca="1">E29*2*1000/E30/E39/E38</f>
-        <v>51.939287331535837</v>
+        <v>47.611013387241179</v>
       </c>
       <c r="F40" t="s">
         <v>16</v>
@@ -10804,7 +11497,7 @@
       <c r="D41" s="124"/>
       <c r="E41">
         <f ca="1">E40+E32</f>
-        <v>63.939287331535837</v>
+        <v>59.611013387241179</v>
       </c>
       <c r="F41" t="s">
         <v>16</v>
@@ -10824,11 +11517,12 @@
     </row>
   </sheetData>
   <mergeCells count="26">
-    <mergeCell ref="A31:F31"/>
     <mergeCell ref="A41:D41"/>
     <mergeCell ref="A38:D38"/>
     <mergeCell ref="A39:D39"/>
     <mergeCell ref="A40:D40"/>
+    <mergeCell ref="A35:D35"/>
+    <mergeCell ref="A36:D36"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="A24:D24"/>
     <mergeCell ref="A25:D25"/>
@@ -10840,8 +11534,6 @@
     <mergeCell ref="A5:D5"/>
     <mergeCell ref="A4:D4"/>
     <mergeCell ref="A6:D6"/>
-    <mergeCell ref="A35:D35"/>
-    <mergeCell ref="A36:D36"/>
     <mergeCell ref="A9:D9"/>
     <mergeCell ref="A10:D10"/>
     <mergeCell ref="A11:D11"/>
@@ -10850,6 +11542,7 @@
     <mergeCell ref="A32:D32"/>
     <mergeCell ref="A34:D34"/>
     <mergeCell ref="A33:D33"/>
+    <mergeCell ref="A31:F31"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -11012,7 +11705,7 @@
       <c r="D17" s="124"/>
       <c r="E17" s="90">
         <f>'тихоходный вал'!E39</f>
-        <v>110</v>
+        <v>120</v>
       </c>
       <c r="F17" t="s">
         <v>378</v>
@@ -11027,7 +11720,7 @@
       <c r="D18" s="124"/>
       <c r="E18">
         <f>E7*2*1000/E8/E17/E16</f>
-        <v>9.2312881291463924</v>
+        <v>8.462014118384193</v>
       </c>
       <c r="F18" t="s">
         <v>16</v>
@@ -11042,7 +11735,7 @@
       <c r="D19" s="124"/>
       <c r="E19">
         <f>E18+E10</f>
-        <v>19.231288129146392</v>
+        <v>18.462014118384193</v>
       </c>
       <c r="F19" t="s">
         <v>16</v>
@@ -11070,6 +11763,298 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{490D1B27-1B6E-4434-A576-709F124EC6EE}">
+  <dimension ref="A2:T11"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="26" width="6.77734375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A2" s="124" t="s">
+        <v>251</v>
+      </c>
+      <c r="B2" s="124"/>
+      <c r="C2" s="124"/>
+      <c r="D2" s="124"/>
+      <c r="E2" s="124"/>
+      <c r="F2" s="124"/>
+      <c r="H2" s="124" t="s">
+        <v>29</v>
+      </c>
+      <c r="I2" s="124"/>
+      <c r="J2" s="124"/>
+      <c r="K2" s="124"/>
+      <c r="L2" s="124"/>
+      <c r="N2" s="124" t="s">
+        <v>252</v>
+      </c>
+      <c r="O2" s="124"/>
+      <c r="P2" s="124"/>
+      <c r="Q2" s="124"/>
+      <c r="R2" s="124"/>
+      <c r="S2" s="124"/>
+    </row>
+    <row r="3" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A3" s="124" t="s">
+        <v>166</v>
+      </c>
+      <c r="B3" s="124"/>
+      <c r="C3" s="124"/>
+      <c r="D3" s="124"/>
+      <c r="E3" s="61">
+        <f>Электродвигатель!$P$53</f>
+        <v>48.741201321892952</v>
+      </c>
+      <c r="F3" t="s">
+        <v>99</v>
+      </c>
+      <c r="H3" s="143" t="s">
+        <v>390</v>
+      </c>
+      <c r="I3" s="143"/>
+      <c r="J3" s="143"/>
+      <c r="K3" s="78">
+        <f>Передача!$D$49</f>
+        <v>2016</v>
+      </c>
+      <c r="L3" s="75" t="s">
+        <v>153</v>
+      </c>
+      <c r="N3" s="124" t="s">
+        <v>166</v>
+      </c>
+      <c r="O3" s="124"/>
+      <c r="P3" s="124"/>
+      <c r="Q3" s="124"/>
+      <c r="R3" s="61">
+        <f ca="1">Электродвигатель!$P$55</f>
+        <v>349.79520039605768</v>
+      </c>
+      <c r="S3" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="4" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A4" s="124" t="s">
+        <v>177</v>
+      </c>
+      <c r="B4" s="124"/>
+      <c r="C4" s="124"/>
+      <c r="D4" s="124"/>
+      <c r="E4">
+        <v>100</v>
+      </c>
+      <c r="F4" t="s">
+        <v>57</v>
+      </c>
+      <c r="G4" t="s">
+        <v>100</v>
+      </c>
+      <c r="H4" s="143" t="s">
+        <v>389</v>
+      </c>
+      <c r="I4" s="143"/>
+      <c r="J4" s="143"/>
+      <c r="K4" s="78">
+        <f>Передача!$D$50</f>
+        <v>734</v>
+      </c>
+      <c r="L4" s="75" t="s">
+        <v>153</v>
+      </c>
+      <c r="N4" s="124" t="s">
+        <v>177</v>
+      </c>
+      <c r="O4" s="124"/>
+      <c r="P4" s="124"/>
+      <c r="Q4" s="124"/>
+      <c r="R4">
+        <v>50</v>
+      </c>
+      <c r="S4" t="s">
+        <v>57</v>
+      </c>
+      <c r="T4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="5" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A5" s="124" t="s">
+        <v>391</v>
+      </c>
+      <c r="B5" s="124"/>
+      <c r="C5" s="124"/>
+      <c r="D5" s="124"/>
+      <c r="E5">
+        <f>E4*SQRT(E3)</f>
+        <v>698.14899070250726</v>
+      </c>
+      <c r="F5" t="s">
+        <v>153</v>
+      </c>
+      <c r="H5" s="143" t="s">
+        <v>388</v>
+      </c>
+      <c r="I5" s="143"/>
+      <c r="J5" s="143"/>
+      <c r="K5" s="78">
+        <f>Передача!$D$51</f>
+        <v>0</v>
+      </c>
+      <c r="L5" s="75" t="s">
+        <v>153</v>
+      </c>
+      <c r="N5" s="124" t="s">
+        <v>391</v>
+      </c>
+      <c r="O5" s="124"/>
+      <c r="P5" s="124"/>
+      <c r="Q5" s="124"/>
+      <c r="R5">
+        <f ca="1">R4*SQRT(R3)</f>
+        <v>935.14063166464132</v>
+      </c>
+      <c r="S5" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="6" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A6" s="124" t="s">
+        <v>177</v>
+      </c>
+      <c r="B6" s="124"/>
+      <c r="C6" s="124"/>
+      <c r="D6" s="124"/>
+      <c r="E6">
+        <v>3</v>
+      </c>
+      <c r="F6" t="s">
+        <v>57</v>
+      </c>
+      <c r="N6" s="124" t="s">
+        <v>177</v>
+      </c>
+      <c r="O6" s="124"/>
+      <c r="P6" s="124"/>
+      <c r="Q6" s="124"/>
+      <c r="R6">
+        <v>3</v>
+      </c>
+      <c r="S6" t="s">
+        <v>57</v>
+      </c>
+      <c r="T6" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="7" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A7" s="124" t="s">
+        <v>387</v>
+      </c>
+      <c r="B7" s="124"/>
+      <c r="C7" s="124"/>
+      <c r="D7" s="124"/>
+      <c r="E7">
+        <v>0</v>
+      </c>
+      <c r="F7" t="s">
+        <v>153</v>
+      </c>
+      <c r="H7" t="s">
+        <v>392</v>
+      </c>
+      <c r="N7" s="124" t="s">
+        <v>387</v>
+      </c>
+      <c r="O7" s="124"/>
+      <c r="P7" s="124"/>
+      <c r="Q7" s="124"/>
+      <c r="R7">
+        <f>R6*K3</f>
+        <v>6048</v>
+      </c>
+      <c r="S7" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="8" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A8" s="124" t="s">
+        <v>383</v>
+      </c>
+      <c r="B8" s="124"/>
+      <c r="C8" s="124"/>
+      <c r="D8" s="124"/>
+      <c r="E8" s="124"/>
+    </row>
+    <row r="9" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A9" s="124" t="s">
+        <v>384</v>
+      </c>
+      <c r="B9" s="124"/>
+      <c r="C9" s="124"/>
+      <c r="D9" s="52">
+        <v>50</v>
+      </c>
+      <c r="E9" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="10" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A10" s="124" t="s">
+        <v>385</v>
+      </c>
+      <c r="B10" s="124"/>
+      <c r="C10" s="124"/>
+      <c r="D10" s="52">
+        <v>50</v>
+      </c>
+      <c r="E10" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="11" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A11" s="124" t="s">
+        <v>386</v>
+      </c>
+      <c r="B11" s="124"/>
+      <c r="C11" s="124"/>
+      <c r="D11" s="52">
+        <v>50.5</v>
+      </c>
+      <c r="E11" t="s">
+        <v>16</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="20">
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="N2:S2"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="N3:Q3"/>
+    <mergeCell ref="H2:L2"/>
+    <mergeCell ref="H3:J3"/>
+    <mergeCell ref="N4:Q4"/>
+    <mergeCell ref="H4:J4"/>
+    <mergeCell ref="H5:J5"/>
+    <mergeCell ref="A8:E8"/>
+    <mergeCell ref="A9:C9"/>
+    <mergeCell ref="A10:C10"/>
+    <mergeCell ref="N5:Q5"/>
+    <mergeCell ref="N7:Q7"/>
+    <mergeCell ref="A7:D7"/>
+    <mergeCell ref="N6:Q6"/>
+    <mergeCell ref="A6:D6"/>
+  </mergeCells>
+  <phoneticPr fontId="3" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B080B891-BABE-48BC-B741-A9DC893B6424}">
   <dimension ref="A2:W23"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -11318,6 +12303,10 @@
       </c>
       <c r="F19" t="s">
         <v>5</v>
+      </c>
+      <c r="I19">
+        <f>1432*30*PI()/1000*42.5/1000</f>
+        <v>5.7359198669242444</v>
       </c>
     </row>
     <row r="20" spans="1:23" x14ac:dyDescent="0.3">
@@ -11422,657 +12411,4 @@
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D8564D3-007A-4908-B584-B11BCC9DA655}">
-  <dimension ref="A1:E80"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" s="124">
-        <v>1</v>
-      </c>
-      <c r="B1">
-        <v>1</v>
-      </c>
-      <c r="D1" s="48"/>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" s="124"/>
-      <c r="B2">
-        <v>1.05</v>
-      </c>
-      <c r="D2" s="48"/>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" s="124">
-        <v>1.1000000000000001</v>
-      </c>
-      <c r="B3">
-        <v>1.1000000000000001</v>
-      </c>
-      <c r="D3" s="48"/>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" s="124"/>
-      <c r="B4">
-        <v>1.1499999999999999</v>
-      </c>
-      <c r="D4" s="48"/>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" s="124">
-        <v>1.2</v>
-      </c>
-      <c r="B5">
-        <v>1.2</v>
-      </c>
-      <c r="D5" s="48"/>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" s="124"/>
-      <c r="B6">
-        <v>1.3</v>
-      </c>
-      <c r="D6" s="48"/>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" s="124">
-        <v>1.4</v>
-      </c>
-      <c r="B7">
-        <v>1.4</v>
-      </c>
-      <c r="D7" s="48"/>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" s="124"/>
-      <c r="B8">
-        <v>1.5</v>
-      </c>
-      <c r="D8" s="48"/>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A9" s="124">
-        <v>1.6</v>
-      </c>
-      <c r="B9">
-        <v>1.6</v>
-      </c>
-      <c r="D9" s="48"/>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A10" s="124"/>
-      <c r="B10">
-        <v>1.7</v>
-      </c>
-      <c r="D10" s="48"/>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A11" s="124">
-        <v>1.8</v>
-      </c>
-      <c r="B11">
-        <v>1.8</v>
-      </c>
-      <c r="D11" s="48"/>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A12" s="124"/>
-      <c r="B12">
-        <v>1.9</v>
-      </c>
-      <c r="D12" s="48"/>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A13" s="124">
-        <v>2</v>
-      </c>
-      <c r="B13">
-        <v>2</v>
-      </c>
-      <c r="D13" s="48"/>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A14" s="124"/>
-      <c r="B14">
-        <v>2.1</v>
-      </c>
-      <c r="D14" s="48"/>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A15" s="124">
-        <v>2.2000000000000002</v>
-      </c>
-      <c r="B15">
-        <v>2.2000000000000002</v>
-      </c>
-      <c r="D15" s="48"/>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A16" s="124"/>
-      <c r="B16">
-        <v>2.4</v>
-      </c>
-      <c r="D16" s="48"/>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A17" s="124">
-        <v>2.5</v>
-      </c>
-      <c r="B17">
-        <v>2.5</v>
-      </c>
-      <c r="D17" s="48"/>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A18" s="124"/>
-      <c r="B18">
-        <v>2.6</v>
-      </c>
-      <c r="D18" s="48"/>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A19" s="124">
-        <v>2.8</v>
-      </c>
-      <c r="B19">
-        <v>2.8</v>
-      </c>
-      <c r="D19" s="48"/>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A20" s="124"/>
-      <c r="B20">
-        <v>3</v>
-      </c>
-      <c r="D20" s="48"/>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A21" s="124">
-        <v>3.2</v>
-      </c>
-      <c r="B21">
-        <v>3.2</v>
-      </c>
-      <c r="D21" s="48"/>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A22" s="124"/>
-      <c r="B22">
-        <v>3.4</v>
-      </c>
-      <c r="D22" s="48"/>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A23" s="124">
-        <v>3.6</v>
-      </c>
-      <c r="B23">
-        <v>3.6</v>
-      </c>
-      <c r="D23" s="48"/>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A24" s="124"/>
-      <c r="B24">
-        <v>3.8</v>
-      </c>
-      <c r="D24" s="48"/>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A25" s="124">
-        <v>4</v>
-      </c>
-      <c r="B25">
-        <v>4</v>
-      </c>
-      <c r="D25" s="48"/>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A26" s="124"/>
-      <c r="B26">
-        <v>4.2</v>
-      </c>
-      <c r="D26" s="48"/>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A27" s="124">
-        <v>4.5</v>
-      </c>
-      <c r="B27">
-        <v>4.5</v>
-      </c>
-      <c r="D27" s="48"/>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A28" s="124"/>
-      <c r="B28">
-        <v>4.8</v>
-      </c>
-      <c r="D28" s="48"/>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A29" s="124">
-        <v>5</v>
-      </c>
-      <c r="B29">
-        <v>5</v>
-      </c>
-      <c r="D29" s="48"/>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A30" s="124"/>
-      <c r="B30">
-        <v>5.3</v>
-      </c>
-      <c r="D30" s="48"/>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A31" s="124">
-        <v>5.6</v>
-      </c>
-      <c r="B31">
-        <v>5.6</v>
-      </c>
-      <c r="D31" s="48"/>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A32" s="124"/>
-      <c r="B32">
-        <v>6</v>
-      </c>
-      <c r="D32" s="48"/>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A33" s="124">
-        <v>6.3</v>
-      </c>
-      <c r="B33">
-        <v>6.3</v>
-      </c>
-      <c r="D33" s="48"/>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A34" s="124"/>
-      <c r="B34">
-        <v>6.7</v>
-      </c>
-      <c r="D34" s="48"/>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A35" s="124">
-        <v>7.1</v>
-      </c>
-      <c r="B35">
-        <v>7.1</v>
-      </c>
-      <c r="D35" s="48"/>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A36" s="124"/>
-      <c r="B36">
-        <v>7.5</v>
-      </c>
-      <c r="D36" s="48"/>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A37" s="124">
-        <v>8</v>
-      </c>
-      <c r="B37">
-        <v>8</v>
-      </c>
-      <c r="D37" s="48"/>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A38" s="124"/>
-      <c r="B38">
-        <v>8.5</v>
-      </c>
-      <c r="D38" s="48"/>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A39" s="124">
-        <v>9</v>
-      </c>
-      <c r="B39">
-        <v>9</v>
-      </c>
-      <c r="D39" s="48"/>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A40" s="124"/>
-      <c r="B40" s="61">
-        <v>9.5</v>
-      </c>
-      <c r="D40" s="48"/>
-      <c r="E40" s="61"/>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A41" s="124">
-        <v>10</v>
-      </c>
-      <c r="B41" s="48">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A42" s="124"/>
-      <c r="B42" s="48">
-        <v>10.5</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A43" s="124">
-        <v>11</v>
-      </c>
-      <c r="B43" s="48">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A44" s="124"/>
-      <c r="B44" s="48">
-        <v>11.5</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A45" s="124">
-        <v>12</v>
-      </c>
-      <c r="B45" s="48">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A46" s="124"/>
-      <c r="B46" s="48">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A47" s="124">
-        <v>14</v>
-      </c>
-      <c r="B47" s="48">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A48" s="124"/>
-      <c r="B48" s="48">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A49" s="124">
-        <v>16</v>
-      </c>
-      <c r="B49" s="48">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A50" s="124"/>
-      <c r="B50" s="48">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A51" s="124">
-        <v>18</v>
-      </c>
-      <c r="B51" s="48">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A52" s="124"/>
-      <c r="B52" s="48">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A53" s="124">
-        <v>20</v>
-      </c>
-      <c r="B53" s="48">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A54" s="124"/>
-      <c r="B54" s="48">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A55" s="124">
-        <v>22</v>
-      </c>
-      <c r="B55" s="48">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A56" s="124"/>
-      <c r="B56" s="48">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A57" s="124">
-        <v>25</v>
-      </c>
-      <c r="B57" s="48">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A58" s="124"/>
-      <c r="B58" s="48">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A59" s="124">
-        <v>28</v>
-      </c>
-      <c r="B59" s="48">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A60" s="124"/>
-      <c r="B60" s="48">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A61" s="124">
-        <v>32</v>
-      </c>
-      <c r="B61" s="48">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A62" s="124"/>
-      <c r="B62" s="48">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A63" s="124">
-        <v>36</v>
-      </c>
-      <c r="B63" s="48">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A64" s="124"/>
-      <c r="B64" s="48">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A65" s="124">
-        <v>40</v>
-      </c>
-      <c r="B65" s="48">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A66" s="124"/>
-      <c r="B66" s="48">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A67" s="124">
-        <v>45</v>
-      </c>
-      <c r="B67" s="48">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A68" s="124"/>
-      <c r="B68" s="48">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A69" s="124">
-        <v>50</v>
-      </c>
-      <c r="B69" s="48">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A70" s="124"/>
-      <c r="B70" s="48">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A71" s="124">
-        <v>56</v>
-      </c>
-      <c r="B71" s="48">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A72" s="124"/>
-      <c r="B72" s="48">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A73" s="124">
-        <v>63</v>
-      </c>
-      <c r="B73" s="48">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A74" s="124"/>
-      <c r="B74" s="48">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A75" s="124">
-        <v>71</v>
-      </c>
-      <c r="B75" s="48">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A76" s="124"/>
-      <c r="B76" s="48">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A77" s="124">
-        <v>80</v>
-      </c>
-      <c r="B77" s="48">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A78" s="124"/>
-      <c r="B78" s="48">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A79" s="124">
-        <v>90</v>
-      </c>
-      <c r="B79" s="48">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="80" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A80" s="124"/>
-      <c r="B80" s="48">
-        <v>95</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="40">
-    <mergeCell ref="A77:A78"/>
-    <mergeCell ref="A79:A80"/>
-    <mergeCell ref="A65:A66"/>
-    <mergeCell ref="A67:A68"/>
-    <mergeCell ref="A69:A70"/>
-    <mergeCell ref="A71:A72"/>
-    <mergeCell ref="A73:A74"/>
-    <mergeCell ref="A75:A76"/>
-    <mergeCell ref="A63:A64"/>
-    <mergeCell ref="A41:A42"/>
-    <mergeCell ref="A43:A44"/>
-    <mergeCell ref="A45:A46"/>
-    <mergeCell ref="A47:A48"/>
-    <mergeCell ref="A49:A50"/>
-    <mergeCell ref="A51:A52"/>
-    <mergeCell ref="A53:A54"/>
-    <mergeCell ref="A55:A56"/>
-    <mergeCell ref="A57:A58"/>
-    <mergeCell ref="A59:A60"/>
-    <mergeCell ref="A61:A62"/>
-    <mergeCell ref="A37:A38"/>
-    <mergeCell ref="A39:A40"/>
-    <mergeCell ref="A25:A26"/>
-    <mergeCell ref="A27:A28"/>
-    <mergeCell ref="A29:A30"/>
-    <mergeCell ref="A31:A32"/>
-    <mergeCell ref="A33:A34"/>
-    <mergeCell ref="A35:A36"/>
-    <mergeCell ref="A23:A24"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="A3:A4"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="A7:A8"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="A13:A14"/>
-    <mergeCell ref="A15:A16"/>
-    <mergeCell ref="A17:A18"/>
-    <mergeCell ref="A19:A20"/>
-    <mergeCell ref="A21:A22"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Check and RPZ start
Sended blueprint to check
Small fixes in it
Added example of RPZ
Start writing RPZ
Upadted natag calculation
Created own blueprint
</commit_message>
<xml_diff>
--- a/Расчёт.xlsx
+++ b/Расчёт.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Professional\Downloads\интститут\курсач детмаш\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E7910F3-46F4-4980-B254-44E390AE7107}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4141E1CB-450A-45A3-B8F3-6E5DC51ED15A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="812" xr2:uid="{7E097F76-7D13-4899-AD2E-10ADA644057F}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="812" firstSheet="1" activeTab="13" xr2:uid="{7E097F76-7D13-4899-AD2E-10ADA644057F}"/>
   </bookViews>
   <sheets>
     <sheet name="Электродвигатель" sheetId="1" r:id="rId1"/>
@@ -1118,9 +1118,6 @@
     <t>Длинна суммарная</t>
   </si>
   <si>
-    <t>H7/u8</t>
-  </si>
-  <si>
     <t>Крышка тихоходного вала</t>
   </si>
   <si>
@@ -1665,6 +1662,9 @@
   </si>
   <si>
     <t>Окржная консольная сила</t>
+  </si>
+  <si>
+    <t>H7/x8</t>
   </si>
 </sst>
 </file>
@@ -3839,7 +3839,7 @@
       <c r="Y19" s="108"/>
       <c r="Z19" s="115"/>
       <c r="AC19" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
     </row>
     <row r="20" spans="9:29" x14ac:dyDescent="0.3">
@@ -4420,7 +4420,7 @@
         <v>169</v>
       </c>
       <c r="AC32" s="65" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="33" spans="2:31" x14ac:dyDescent="0.3">
@@ -4500,7 +4500,7 @@
         <v>179</v>
       </c>
       <c r="AC34" s="65" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="35" spans="2:31" x14ac:dyDescent="0.3">
@@ -4540,7 +4540,7 @@
         <v>67</v>
       </c>
       <c r="AC35" s="96" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
     </row>
     <row r="36" spans="2:31" x14ac:dyDescent="0.3">
@@ -4623,7 +4623,7 @@
     </row>
     <row r="37" spans="2:31" x14ac:dyDescent="0.3">
       <c r="AC37" s="65" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="38" spans="2:31" x14ac:dyDescent="0.3">
@@ -4920,7 +4920,7 @@
         <v>198</v>
       </c>
       <c r="AC42" s="65" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
     </row>
     <row r="43" spans="2:31" x14ac:dyDescent="0.3">
@@ -5002,7 +5002,7 @@
         <v>177</v>
       </c>
       <c r="AC43" s="65" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="44" spans="2:31" x14ac:dyDescent="0.3">
@@ -5075,7 +5075,7 @@
         <v>0</v>
       </c>
       <c r="AA44" s="141" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="AB44" s="142"/>
       <c r="AC44" s="71" t="s">
@@ -5232,7 +5232,7 @@
         <v>0.75835111197354876</v>
       </c>
       <c r="AC46" s="132" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="AD46" s="132"/>
       <c r="AE46" s="132"/>
@@ -5267,7 +5267,7 @@
         <v>57</v>
       </c>
       <c r="AC47" s="71" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
     </row>
     <row r="48" spans="2:31" x14ac:dyDescent="0.3">
@@ -5309,7 +5309,7 @@
         <v>298</v>
       </c>
       <c r="AC48" s="71" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
     </row>
     <row r="49" spans="2:29" x14ac:dyDescent="0.3">
@@ -5345,7 +5345,7 @@
         <v>300</v>
       </c>
       <c r="AC49" s="71" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
     </row>
     <row r="50" spans="2:29" x14ac:dyDescent="0.3">
@@ -5373,7 +5373,7 @@
         <v>300</v>
       </c>
       <c r="AC50" s="71" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
     </row>
     <row r="51" spans="2:29" x14ac:dyDescent="0.3">
@@ -5403,7 +5403,7 @@
       </c>
       <c r="M51" s="108"/>
       <c r="N51" s="145" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="O51" s="145"/>
       <c r="P51" s="108" t="s">
@@ -5424,7 +5424,7 @@
         <v>57</v>
       </c>
       <c r="AC51" s="71" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
     </row>
     <row r="52" spans="2:29" x14ac:dyDescent="0.3">
@@ -5478,7 +5478,7 @@
         <v>315</v>
       </c>
       <c r="AC52" s="71" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
     </row>
     <row r="53" spans="2:29" x14ac:dyDescent="0.3">
@@ -5528,7 +5528,7 @@
         <v>206</v>
       </c>
       <c r="AC53" s="71" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
     </row>
     <row r="54" spans="2:29" x14ac:dyDescent="0.3">
@@ -5578,7 +5578,7 @@
         <v>302</v>
       </c>
       <c r="AC54" s="71" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="55" spans="2:29" x14ac:dyDescent="0.3">
@@ -5629,7 +5629,7 @@
         <v>205</v>
       </c>
       <c r="AC55" s="71" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
     </row>
     <row r="56" spans="2:29" x14ac:dyDescent="0.3">
@@ -5992,7 +5992,7 @@
   <sheetData>
     <row r="1" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="C1">
         <f ca="1">Электродвигатель!P58</f>
@@ -6054,7 +6054,7 @@
     </row>
     <row r="4" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="C4">
         <f>Электродвигатель!F53</f>
@@ -6066,7 +6066,7 @@
       <c r="F4" s="16"/>
       <c r="H4" s="16"/>
       <c r="O4" s="110" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="P4" s="110"/>
       <c r="Q4" s="110"/>
@@ -6082,14 +6082,14 @@
     <row r="5" spans="1:21" x14ac:dyDescent="0.3">
       <c r="H5" s="16"/>
       <c r="I5" s="107" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="J5" s="108"/>
       <c r="K5" s="108"/>
       <c r="L5" s="115"/>
       <c r="M5" s="1"/>
       <c r="O5" s="132" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="P5" s="132"/>
       <c r="Q5" s="132"/>
@@ -6107,7 +6107,7 @@
     <row r="6" spans="1:21" x14ac:dyDescent="0.3">
       <c r="H6" s="48"/>
       <c r="I6" s="102" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="J6" s="16"/>
       <c r="K6" s="1"/>
@@ -6138,14 +6138,14 @@
       <c r="G7" s="1"/>
       <c r="H7" s="48"/>
       <c r="I7" s="7" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="J7" s="1"/>
       <c r="K7" s="1"/>
       <c r="L7" s="3"/>
       <c r="M7" s="1"/>
       <c r="O7" s="132" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="P7" s="132"/>
       <c r="Q7" s="132"/>
@@ -6170,16 +6170,16 @@
       <c r="G8" s="1"/>
       <c r="H8" s="48"/>
       <c r="I8" s="7" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="J8" s="1"/>
       <c r="K8" s="1" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="L8" s="3"/>
       <c r="M8" s="1"/>
       <c r="O8" s="132" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="P8" s="132"/>
       <c r="Q8" s="132"/>
@@ -6208,16 +6208,16 @@
       <c r="G9" s="1"/>
       <c r="H9" s="48"/>
       <c r="I9" s="7" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="J9" s="1"/>
       <c r="K9" s="1" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="L9" s="3"/>
       <c r="M9" s="1"/>
       <c r="O9" s="132" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="P9" s="132"/>
       <c r="Q9" s="132"/>
@@ -6240,14 +6240,14 @@
       </c>
       <c r="G10" s="1"/>
       <c r="I10" s="7" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="J10" s="1"/>
       <c r="K10" s="1"/>
       <c r="L10" s="3"/>
       <c r="M10" s="1"/>
       <c r="O10" s="132" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="P10" s="132"/>
       <c r="Q10" s="132"/>
@@ -6259,7 +6259,7 @@
         <v>16</v>
       </c>
       <c r="U10" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
     </row>
     <row r="11" spans="1:21" x14ac:dyDescent="0.3">
@@ -6277,16 +6277,16 @@
       </c>
       <c r="G11" s="1"/>
       <c r="I11" s="7" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="J11" s="1"/>
       <c r="K11" s="1" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="L11" s="3"/>
       <c r="M11" s="1"/>
       <c r="O11" s="132" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="P11" s="132"/>
       <c r="Q11" s="132"/>
@@ -6298,7 +6298,7 @@
         <v>16</v>
       </c>
       <c r="U11" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
     </row>
     <row r="12" spans="1:21" x14ac:dyDescent="0.3">
@@ -6316,7 +6316,7 @@
       </c>
       <c r="G12" s="1"/>
       <c r="I12" s="7" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="J12" s="1">
         <v>52</v>
@@ -6327,7 +6327,7 @@
       <c r="L12" s="3"/>
       <c r="M12" s="1"/>
       <c r="O12" s="132" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="P12" s="132"/>
       <c r="Q12" s="132"/>
@@ -6339,7 +6339,7 @@
         <v>16</v>
       </c>
       <c r="U12" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.3">
@@ -6368,7 +6368,7 @@
       <c r="L13" s="3"/>
       <c r="M13" s="1"/>
       <c r="O13" s="132" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="P13" s="132"/>
       <c r="Q13" s="132"/>
@@ -6380,7 +6380,7 @@
         <v>16</v>
       </c>
       <c r="U13" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.3">
@@ -6409,7 +6409,7 @@
       <c r="L14" s="3"/>
       <c r="M14" s="1"/>
       <c r="O14" s="132" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="P14" s="132"/>
       <c r="Q14" s="132"/>
@@ -6417,7 +6417,7 @@
       <c r="S14" s="132"/>
       <c r="T14" s="132"/>
       <c r="U14" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.3">
@@ -6435,7 +6435,7 @@
       </c>
       <c r="G15" s="1"/>
       <c r="I15" s="7" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="J15" s="25">
         <v>8</v>
@@ -6446,7 +6446,7 @@
       <c r="L15" s="3"/>
       <c r="M15" s="1"/>
       <c r="O15" s="132" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="P15" s="132"/>
       <c r="Q15" s="132"/>
@@ -6474,7 +6474,7 @@
       </c>
       <c r="G16" s="1"/>
       <c r="I16" s="106" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="J16" s="25">
         <v>0.5</v>
@@ -6485,7 +6485,7 @@
       <c r="L16" s="3"/>
       <c r="M16" s="1"/>
       <c r="O16" s="132" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="P16" s="132"/>
       <c r="Q16" s="132"/>
@@ -6508,11 +6508,11 @@
         <v>1309</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="G17" s="1"/>
       <c r="I17" s="104" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="J17" s="1">
         <v>25</v>
@@ -6523,7 +6523,7 @@
       <c r="L17" s="3"/>
       <c r="M17" s="1"/>
       <c r="O17" s="132" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="P17" s="132"/>
       <c r="Q17" s="132"/>
@@ -6550,19 +6550,19 @@
       </c>
       <c r="G18" s="1"/>
       <c r="I18" s="7" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="J18" s="1">
         <f>0.2*J12*J12*J12</f>
         <v>28121.600000000002</v>
       </c>
       <c r="K18" s="25" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L18" s="3"/>
       <c r="M18" s="1"/>
       <c r="O18" s="132" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="P18" s="132"/>
       <c r="Q18" s="132"/>
@@ -6589,7 +6589,7 @@
       </c>
       <c r="G19" s="1"/>
       <c r="I19" s="105" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="J19" s="1">
         <v>1.3</v>
@@ -6598,7 +6598,7 @@
       <c r="L19" s="3"/>
       <c r="M19" s="1"/>
       <c r="O19" s="132" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="P19" s="132"/>
       <c r="Q19" s="132"/>
@@ -6613,7 +6613,7 @@
     </row>
     <row r="20" spans="2:20" x14ac:dyDescent="0.3">
       <c r="B20" s="109" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="C20" s="110"/>
       <c r="D20" s="110"/>
@@ -6625,7 +6625,7 @@
       </c>
       <c r="G20" s="1"/>
       <c r="I20" s="105" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="J20" s="1">
         <f>(J13+J12)/2</f>
@@ -6637,7 +6637,7 @@
       <c r="L20" s="3"/>
       <c r="M20" s="1"/>
       <c r="O20" s="132" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="P20" s="132"/>
       <c r="Q20" s="132"/>
@@ -6652,7 +6652,7 @@
     </row>
     <row r="21" spans="2:20" x14ac:dyDescent="0.3">
       <c r="B21" s="109" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="C21" s="110"/>
       <c r="D21" s="110"/>
@@ -6675,7 +6675,7 @@
       </c>
       <c r="L21" s="3"/>
       <c r="O21" s="132" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="P21" s="132"/>
       <c r="Q21" s="132"/>
@@ -6690,21 +6690,21 @@
     </row>
     <row r="22" spans="2:20" x14ac:dyDescent="0.3">
       <c r="B22" s="7" t="s">
+        <v>470</v>
+      </c>
+      <c r="C22" s="7" t="s">
+        <v>472</v>
+      </c>
+      <c r="D22" s="7" t="s">
         <v>471</v>
       </c>
-      <c r="C22" s="7" t="s">
-        <v>473</v>
-      </c>
-      <c r="D22" s="7" t="s">
-        <v>472</v>
-      </c>
       <c r="E22" s="12" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="F22" s="3"/>
       <c r="G22" s="1"/>
       <c r="I22" s="7" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="J22" s="1" t="b">
         <f ca="1">C1/J18*1000&lt;J17</f>
@@ -6713,7 +6713,7 @@
       <c r="K22" s="1"/>
       <c r="L22" s="3"/>
       <c r="O22" s="132" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="P22" s="132"/>
       <c r="Q22" s="132"/>
@@ -6736,7 +6736,7 @@
       </c>
       <c r="F23" s="3"/>
       <c r="I23" s="106" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="J23" s="1" t="b">
         <f ca="1">2*C1*J19/J20/J15/J21/J24&lt;J25</f>
@@ -6745,7 +6745,7 @@
       <c r="K23" s="1"/>
       <c r="L23" s="3"/>
       <c r="O23" s="132" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="P23" s="132"/>
       <c r="Q23" s="132"/>
@@ -6772,7 +6772,7 @@
       <c r="K24" s="1"/>
       <c r="L24" s="3"/>
       <c r="O24" s="132" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="P24" s="132"/>
       <c r="Q24" s="132"/>
@@ -6791,7 +6791,7 @@
       <c r="E25" s="4"/>
       <c r="F25" s="5"/>
       <c r="I25" s="7" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="J25" s="1">
         <f>0.4*240</f>
@@ -6800,7 +6800,7 @@
       <c r="K25" s="1"/>
       <c r="L25" s="3"/>
       <c r="O25" s="132" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="P25" s="132"/>
       <c r="Q25" s="132"/>
@@ -6824,7 +6824,7 @@
       <c r="K26" s="4"/>
       <c r="L26" s="5"/>
       <c r="O26" s="132" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="P26" s="132"/>
       <c r="Q26" s="132"/>
@@ -6839,7 +6839,7 @@
     </row>
     <row r="27" spans="2:20" x14ac:dyDescent="0.3">
       <c r="O27" s="132" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="P27" s="132"/>
       <c r="Q27" s="132"/>
@@ -6854,7 +6854,7 @@
     </row>
     <row r="28" spans="2:20" x14ac:dyDescent="0.3">
       <c r="O28" s="132" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="P28" s="132"/>
       <c r="Q28" s="132"/>
@@ -6869,7 +6869,7 @@
     </row>
     <row r="29" spans="2:20" x14ac:dyDescent="0.3">
       <c r="O29" s="132" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="P29" s="132"/>
       <c r="Q29" s="132"/>
@@ -6884,7 +6884,7 @@
     </row>
     <row r="31" spans="2:20" x14ac:dyDescent="0.3">
       <c r="H31" s="132" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="I31" s="132"/>
       <c r="J31" s="132"/>
@@ -6894,7 +6894,7 @@
         <v>10000</v>
       </c>
       <c r="O31" s="132" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="P31" s="132"/>
       <c r="Q31" s="132"/>
@@ -6909,7 +6909,7 @@
     </row>
     <row r="32" spans="2:20" x14ac:dyDescent="0.3">
       <c r="H32" s="132" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="I32" s="132"/>
       <c r="J32" s="132"/>
@@ -6919,7 +6919,7 @@
         <v>0.9</v>
       </c>
       <c r="O32" s="132" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="P32" s="132"/>
       <c r="Q32" s="132"/>
@@ -6934,7 +6934,7 @@
     </row>
     <row r="33" spans="8:20" x14ac:dyDescent="0.3">
       <c r="H33" s="132" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="I33" s="132"/>
       <c r="J33" s="132"/>
@@ -6945,7 +6945,7 @@
     </row>
     <row r="34" spans="8:20" x14ac:dyDescent="0.3">
       <c r="H34" s="132" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="I34" s="132"/>
       <c r="J34" s="132"/>
@@ -6957,7 +6957,7 @@
     </row>
     <row r="35" spans="8:20" x14ac:dyDescent="0.3">
       <c r="H35" s="132" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="I35" s="132"/>
       <c r="J35" s="132"/>
@@ -6967,7 +6967,7 @@
         <v>2.66</v>
       </c>
       <c r="O35" s="132" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="P35" s="132"/>
       <c r="Q35" s="132"/>
@@ -6976,7 +6976,7 @@
     </row>
     <row r="36" spans="8:20" x14ac:dyDescent="0.3">
       <c r="H36" s="132" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="I36" s="132"/>
       <c r="J36" s="132"/>
@@ -6985,7 +6985,7 @@
         <v>1</v>
       </c>
       <c r="O36" s="132" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="P36" s="132"/>
       <c r="Q36" s="132"/>
@@ -6994,7 +6994,7 @@
     </row>
     <row r="37" spans="8:20" x14ac:dyDescent="0.3">
       <c r="H37" s="132" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="I37" s="132"/>
       <c r="J37" s="132"/>
@@ -7003,7 +7003,7 @@
         <v>1.6</v>
       </c>
       <c r="O37" s="132" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="P37" s="132"/>
       <c r="Q37" s="132"/>
@@ -7018,7 +7018,7 @@
     </row>
     <row r="38" spans="8:20" x14ac:dyDescent="0.3">
       <c r="H38" s="132" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="I38" s="132"/>
       <c r="J38" s="132"/>
@@ -7027,7 +7027,7 @@
         <v>1</v>
       </c>
       <c r="O38" s="132" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="P38" s="132"/>
       <c r="Q38" s="132"/>
@@ -7042,7 +7042,7 @@
     </row>
     <row r="39" spans="8:20" x14ac:dyDescent="0.3">
       <c r="H39" s="132" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="I39" s="132"/>
       <c r="J39" s="132"/>
@@ -7053,7 +7053,7 @@
     </row>
     <row r="40" spans="8:20" x14ac:dyDescent="0.3">
       <c r="H40" s="132" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="I40" s="132"/>
       <c r="J40" s="132"/>
@@ -7063,7 +7063,7 @@
         <v>22</v>
       </c>
       <c r="O40" s="132" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="P40" s="132"/>
       <c r="Q40" s="132"/>
@@ -7072,7 +7072,7 @@
     </row>
     <row r="41" spans="8:20" x14ac:dyDescent="0.3">
       <c r="H41" s="132" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="I41" s="132"/>
       <c r="J41" s="132"/>
@@ -7082,7 +7082,7 @@
         <v>3</v>
       </c>
       <c r="O41" s="132" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="P41" s="132"/>
       <c r="Q41" s="132"/>
@@ -7097,7 +7097,7 @@
     </row>
     <row r="42" spans="8:20" x14ac:dyDescent="0.3">
       <c r="H42" s="132" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="I42" s="132"/>
       <c r="J42" s="132"/>
@@ -7106,7 +7106,7 @@
         <v>0.63</v>
       </c>
       <c r="O42" s="132" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="P42" s="132"/>
       <c r="Q42" s="132"/>
@@ -7119,7 +7119,7 @@
     </row>
     <row r="43" spans="8:20" x14ac:dyDescent="0.3">
       <c r="O43" s="132" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="P43" s="132"/>
       <c r="Q43" s="132"/>
@@ -7138,7 +7138,7 @@
     </row>
     <row r="45" spans="8:20" x14ac:dyDescent="0.3">
       <c r="O45" s="132" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="P45" s="132"/>
       <c r="Q45" s="132"/>
@@ -7153,7 +7153,7 @@
     </row>
     <row r="46" spans="8:20" x14ac:dyDescent="0.3">
       <c r="O46" s="132" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="P46" s="132"/>
       <c r="Q46" s="132"/>
@@ -7168,7 +7168,7 @@
     </row>
     <row r="47" spans="8:20" x14ac:dyDescent="0.3">
       <c r="O47" s="132" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="P47" s="132"/>
       <c r="Q47" s="132"/>
@@ -7183,13 +7183,13 @@
     </row>
     <row r="48" spans="8:20" x14ac:dyDescent="0.3">
       <c r="O48" s="132" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="P48" s="132"/>
     </row>
     <row r="49" spans="15:21" x14ac:dyDescent="0.3">
       <c r="O49" s="132" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="P49" s="132"/>
       <c r="Q49" s="132"/>
@@ -7204,7 +7204,7 @@
     </row>
     <row r="50" spans="15:21" x14ac:dyDescent="0.3">
       <c r="O50" s="132" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="P50" s="132"/>
       <c r="Q50" s="132"/>
@@ -7225,19 +7225,19 @@
         <v>327</v>
       </c>
       <c r="Q52" t="s">
+        <v>416</v>
+      </c>
+      <c r="R52" t="s">
+        <v>422</v>
+      </c>
+      <c r="S52" t="s">
         <v>417</v>
       </c>
-      <c r="R52" t="s">
-        <v>423</v>
-      </c>
-      <c r="S52" t="s">
+      <c r="T52" t="s">
+        <v>419</v>
+      </c>
+      <c r="U52" t="s">
         <v>418</v>
-      </c>
-      <c r="T52" t="s">
-        <v>420</v>
-      </c>
-      <c r="U52" t="s">
-        <v>419</v>
       </c>
     </row>
     <row r="53" spans="15:21" x14ac:dyDescent="0.3">
@@ -7266,7 +7266,7 @@
     </row>
     <row r="55" spans="15:21" x14ac:dyDescent="0.3">
       <c r="O55" s="132" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="P55" s="132"/>
       <c r="Q55" s="132"/>
@@ -7292,12 +7292,12 @@
       </c>
       <c r="T56" s="132"/>
       <c r="U56" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="57" spans="15:21" x14ac:dyDescent="0.3">
       <c r="O57" s="132" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="P57" s="132"/>
       <c r="Q57" s="132"/>
@@ -7338,6 +7338,7 @@
     <mergeCell ref="O31:R31"/>
     <mergeCell ref="O32:R32"/>
     <mergeCell ref="O36:S36"/>
+    <mergeCell ref="O37:R37"/>
     <mergeCell ref="H42:K42"/>
     <mergeCell ref="H36:K36"/>
     <mergeCell ref="H37:K37"/>
@@ -7361,7 +7362,6 @@
     <mergeCell ref="O43:R43"/>
     <mergeCell ref="S43:T43"/>
     <mergeCell ref="O45:R45"/>
-    <mergeCell ref="O37:R37"/>
     <mergeCell ref="O38:R38"/>
     <mergeCell ref="O40:S40"/>
     <mergeCell ref="O41:R41"/>
@@ -7417,12 +7417,12 @@
   <sheetData>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="D3">
         <v>0.3</v>
@@ -7434,30 +7434,30 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
+        <v>497</v>
+      </c>
+      <c r="D4" t="s">
         <v>498</v>
       </c>
-      <c r="D4" t="s">
-        <v>499</v>
-      </c>
       <c r="E4" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="F4">
         <f>0.6*34.5</f>
         <v>20.7</v>
       </c>
       <c r="G4" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="B7" s="60">
         <f>Электродвигатель!P52</f>
@@ -8308,10 +8308,10 @@
         <v>286</v>
       </c>
       <c r="H11" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="I11" s="4" t="s">
         <v>425</v>
-      </c>
-      <c r="I11" s="4" t="s">
-        <v>426</v>
       </c>
       <c r="J11" s="12" t="s">
         <v>284</v>
@@ -8323,10 +8323,10 @@
         <v>286</v>
       </c>
       <c r="M11" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="N11" s="4" t="s">
         <v>425</v>
-      </c>
-      <c r="N11" s="4" t="s">
-        <v>426</v>
       </c>
       <c r="O11" s="4" t="s">
         <v>284</v>
@@ -8338,10 +8338,10 @@
         <v>286</v>
       </c>
       <c r="R11" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="S11" s="4" t="s">
         <v>425</v>
-      </c>
-      <c r="S11" s="4" t="s">
-        <v>426</v>
       </c>
     </row>
     <row r="12" spans="1:20" x14ac:dyDescent="0.3">
@@ -9915,7 +9915,7 @@
     </row>
     <row r="19" spans="1:20" x14ac:dyDescent="0.3">
       <c r="H19" s="107" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="I19" s="108"/>
       <c r="J19" s="108"/>
@@ -9924,7 +9924,7 @@
       </c>
       <c r="L19" s="6"/>
       <c r="P19" s="107" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="Q19" s="108"/>
       <c r="R19" s="108"/>
@@ -10009,7 +10009,7 @@
     </row>
     <row r="23" spans="1:20" x14ac:dyDescent="0.3">
       <c r="H23" s="109" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="I23" s="110"/>
       <c r="J23" s="110"/>
@@ -10021,7 +10021,7 @@
         <v>4</v>
       </c>
       <c r="P23" s="109" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="Q23" s="110"/>
       <c r="R23" s="110"/>
@@ -10035,7 +10035,7 @@
     </row>
     <row r="24" spans="1:20" x14ac:dyDescent="0.3">
       <c r="H24" s="119" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="I24" s="120"/>
       <c r="J24" s="120"/>
@@ -10047,7 +10047,7 @@
         <v>4</v>
       </c>
       <c r="P24" s="119" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="Q24" s="120"/>
       <c r="R24" s="120"/>
@@ -10378,13 +10378,13 @@
     </row>
     <row r="16" spans="2:10" x14ac:dyDescent="0.3">
       <c r="C16" s="132" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="D16" s="132"/>
       <c r="E16" s="132"/>
       <c r="F16" s="132"/>
       <c r="G16" s="132" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="H16" s="132"/>
       <c r="I16" s="132"/>
@@ -10495,7 +10495,7 @@
         <v>6</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="G21" s="12">
         <f ca="1">G18+2*F14</f>
@@ -10507,7 +10507,7 @@
         <v>6</v>
       </c>
       <c r="J21" s="5" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.3">
@@ -11965,7 +11965,7 @@
         <v>251</v>
       </c>
       <c r="T38" s="75" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="U38" s="156" t="s">
         <v>159</v>
@@ -12865,7 +12865,7 @@
       <c r="K10" s="132"/>
       <c r="L10" s="132"/>
       <c r="M10" s="52">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N10" s="25" t="s">
         <v>221</v>
@@ -12979,7 +12979,7 @@
       <c r="L13" s="132"/>
       <c r="M13">
         <f ca="1">2000*M10*M9/(PI()*E19*E19*M12*M11)</f>
-        <v>46.98792560548906</v>
+        <v>62.650567473985404</v>
       </c>
       <c r="N13" t="s">
         <v>223</v>
@@ -13006,7 +13006,7 @@
       <c r="L14" s="132"/>
       <c r="M14">
         <f ca="1">1000*M13*E19*(X10/X8+Z10/Z8)</f>
-        <v>46.673015345699184</v>
+        <v>62.230687127598905</v>
       </c>
       <c r="N14" t="s">
         <v>232</v>
@@ -13033,7 +13033,7 @@
       <c r="L15" s="132"/>
       <c r="M15">
         <f>5.5*(E20+'тихоходный вал'!E8)</f>
-        <v>13.200000000000003</v>
+        <v>17.600000000000001</v>
       </c>
       <c r="N15" t="s">
         <v>232</v>
@@ -13085,7 +13085,7 @@
       <c r="L17" s="132"/>
       <c r="M17" s="25">
         <f ca="1">SUM(M14:M16)</f>
-        <v>59.873015345699187</v>
+        <v>79.830687127598907</v>
       </c>
       <c r="N17" t="s">
         <v>232</v>
@@ -13138,7 +13138,7 @@
       <c r="L19" s="132"/>
       <c r="M19" s="88">
         <f ca="1">M18+M15</f>
-        <v>336.02186948853614</v>
+        <v>340.42186948853617</v>
       </c>
       <c r="N19" t="s">
         <v>232</v>
@@ -13158,7 +13158,7 @@
         <v>232</v>
       </c>
       <c r="M20" s="92" t="s">
-        <v>348</v>
+        <v>507</v>
       </c>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.3">
@@ -13181,10 +13181,10 @@
       <c r="K21" s="132"/>
       <c r="L21" s="132"/>
       <c r="M21">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="N21">
-        <v>108</v>
+        <v>154</v>
       </c>
       <c r="O21" t="s">
         <v>232</v>
@@ -13220,8 +13220,8 @@
       <c r="K23" s="132"/>
       <c r="L23" s="132"/>
       <c r="M23">
-        <f ca="1">PI()*E19*M12*(M21-M15)*M22/1000</f>
-        <v>104.00430975268226</v>
+        <f ca="1">PI()*E19*M12*(N21-M15)*M22/1000</f>
+        <v>268.67780019442915</v>
       </c>
       <c r="N23" t="s">
         <v>4</v>
@@ -13603,7 +13603,7 @@
       <c r="C8" s="132"/>
       <c r="D8" s="132"/>
       <c r="E8" s="52">
-        <v>0.8</v>
+        <v>1.6</v>
       </c>
       <c r="F8" t="s">
         <v>232</v>
@@ -13623,7 +13623,7 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="132" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="B10" s="132"/>
       <c r="C10" s="132"/>
@@ -13635,7 +13635,7 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="132" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B11" s="132"/>
       <c r="C11" s="132"/>
@@ -13655,7 +13655,7 @@
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="132" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="B19" s="132"/>
       <c r="C19" s="132"/>
@@ -13664,23 +13664,23 @@
         <v>1.4</v>
       </c>
       <c r="F19" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="132" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="B20" s="132"/>
       <c r="C20" s="132"/>
       <c r="D20" s="132"/>
       <c r="E20" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" s="132" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="B26" s="132"/>
       <c r="C26" s="132"/>
@@ -13689,12 +13689,12 @@
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" s="132" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="B28" s="132"/>
       <c r="C28" s="132"/>
@@ -13732,7 +13732,7 @@
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" s="132" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B31" s="132"/>
       <c r="C31" s="132"/>
@@ -13742,7 +13742,7 @@
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" s="132" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="B32" s="132"/>
       <c r="C32" s="132"/>
@@ -13756,7 +13756,7 @@
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A33" s="132" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B33" s="132"/>
       <c r="C33" s="132"/>
@@ -13770,7 +13770,7 @@
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A34" s="132" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="B34" s="132"/>
       <c r="C34" s="132"/>
@@ -13798,7 +13798,7 @@
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A36" s="132" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="B36" s="132"/>
       <c r="C36" s="132"/>
@@ -13818,7 +13818,7 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38" s="132" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="B38" s="132"/>
       <c r="C38" s="132"/>
@@ -13833,7 +13833,7 @@
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A39" s="132" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="B39" s="132"/>
       <c r="C39" s="132"/>
@@ -13842,7 +13842,7 @@
         <v>120</v>
       </c>
       <c r="F39" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="G39" t="s">
         <v>100</v>
@@ -13850,7 +13850,7 @@
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A40" s="132" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="B40" s="132"/>
       <c r="C40" s="132"/>
@@ -13935,7 +13935,7 @@
   <sheetData>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="132" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="B6" s="132"/>
       <c r="C6" s="132"/>
@@ -13973,7 +13973,7 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="132" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B9" s="132"/>
       <c r="C9" s="132"/>
@@ -13983,7 +13983,7 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="132" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="B10" s="132"/>
       <c r="C10" s="132"/>
@@ -13997,7 +13997,7 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="132" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B11" s="132"/>
       <c r="C11" s="132"/>
@@ -14011,7 +14011,7 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="132" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="B12" s="132"/>
       <c r="C12" s="132"/>
@@ -14039,7 +14039,7 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="132" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="B14" s="132"/>
       <c r="C14" s="132"/>
@@ -14059,7 +14059,7 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="132" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="B16" s="132"/>
       <c r="C16" s="132"/>
@@ -14074,7 +14074,7 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="132" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="B17" s="132"/>
       <c r="C17" s="132"/>
@@ -14084,12 +14084,12 @@
         <v>120</v>
       </c>
       <c r="F17" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="132" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="B18" s="132"/>
       <c r="C18" s="132"/>
@@ -14201,7 +14201,7 @@
         <v>310</v>
       </c>
       <c r="H3" s="153" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="I3" s="153"/>
       <c r="J3" s="153"/>
@@ -14243,7 +14243,7 @@
         <v>100</v>
       </c>
       <c r="H4" s="153" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="I4" s="153"/>
       <c r="J4" s="153"/>
@@ -14272,7 +14272,7 @@
     </row>
     <row r="5" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A5" s="132" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="B5" s="132"/>
       <c r="C5" s="132"/>
@@ -14285,7 +14285,7 @@
         <v>152</v>
       </c>
       <c r="H5" s="153" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="I5" s="153"/>
       <c r="J5" s="153"/>
@@ -14297,7 +14297,7 @@
         <v>152</v>
       </c>
       <c r="N5" s="132" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="O5" s="132"/>
       <c r="P5" s="132"/>
@@ -14332,7 +14332,7 @@
     </row>
     <row r="7" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A7" s="132" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="B7" s="132"/>
       <c r="C7" s="132"/>
@@ -14344,10 +14344,10 @@
         <v>152</v>
       </c>
       <c r="H7" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="N7" s="132" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="O7" s="132"/>
       <c r="P7" s="132"/>
@@ -14364,7 +14364,7 @@
     </row>
     <row r="8" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A8" s="132" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="B8" s="132"/>
       <c r="C8" s="132"/>
@@ -14372,7 +14372,7 @@
       <c r="E8" s="132"/>
       <c r="F8" s="132"/>
       <c r="N8" s="132" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="O8" s="132"/>
       <c r="P8" s="132"/>
@@ -14382,7 +14382,7 @@
     </row>
     <row r="9" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A9" s="132" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="B9" s="132"/>
       <c r="C9" s="132"/>
@@ -14394,7 +14394,7 @@
         <v>16</v>
       </c>
       <c r="N9" s="132" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="O9" s="132"/>
       <c r="P9" s="132"/>
@@ -14408,7 +14408,7 @@
     </row>
     <row r="10" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A10" s="132" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="B10" s="132"/>
       <c r="C10" s="132"/>
@@ -14420,7 +14420,7 @@
         <v>16</v>
       </c>
       <c r="N10" s="132" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="O10" s="132"/>
       <c r="P10" s="132"/>
@@ -14434,7 +14434,7 @@
     </row>
     <row r="11" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A11" s="132" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="B11" s="132"/>
       <c r="C11" s="132"/>
@@ -14446,7 +14446,7 @@
         <v>16</v>
       </c>
       <c r="N11" s="132" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="O11" s="132"/>
       <c r="P11" s="132"/>
@@ -14468,7 +14468,7 @@
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A13" s="132" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="B13" s="132"/>
       <c r="C13" s="132"/>
@@ -14476,7 +14476,7 @@
       <c r="E13" s="132"/>
       <c r="F13" s="132"/>
       <c r="N13" s="132" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="O13" s="132"/>
       <c r="P13" s="132"/>
@@ -14486,7 +14486,7 @@
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A14" s="132" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B14" s="132"/>
       <c r="C14" s="132"/>
@@ -14499,7 +14499,7 @@
         <v>152</v>
       </c>
       <c r="N14" s="132" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="O14" s="132"/>
       <c r="P14" s="132"/>
@@ -14514,7 +14514,7 @@
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A15" s="132" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="B15" s="132"/>
       <c r="C15" s="132"/>
@@ -14527,7 +14527,7 @@
         <v>152</v>
       </c>
       <c r="N15" s="132" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="O15" s="132"/>
       <c r="P15" s="132"/>
@@ -14542,7 +14542,7 @@
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A16" s="132" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="B16" s="132"/>
       <c r="C16" s="132"/>
@@ -14555,7 +14555,7 @@
         <v>152</v>
       </c>
       <c r="N16" s="132" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="O16" s="132"/>
       <c r="P16" s="132"/>
@@ -14570,7 +14570,7 @@
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A17" s="132" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="B17" s="132"/>
       <c r="C17" s="132"/>
@@ -14583,7 +14583,7 @@
         <v>152</v>
       </c>
       <c r="N17" s="132" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="O17" s="132"/>
       <c r="P17" s="132"/>
@@ -14598,7 +14598,7 @@
     </row>
     <row r="18" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A18" s="132" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="B18" s="132"/>
       <c r="C18" s="132"/>
@@ -14611,7 +14611,7 @@
         <v>152</v>
       </c>
       <c r="N18" s="132" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="O18" s="132"/>
       <c r="P18" s="132"/>
@@ -14626,7 +14626,7 @@
     </row>
     <row r="19" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A19" s="132" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="B19" s="132"/>
       <c r="C19" s="132"/>
@@ -14639,7 +14639,7 @@
         <v>152</v>
       </c>
       <c r="N19" s="132" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="O19" s="132"/>
       <c r="P19" s="132"/>
@@ -14654,7 +14654,7 @@
     </row>
     <row r="20" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A20" s="132" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="B20" s="132"/>
       <c r="C20" s="132"/>
@@ -14667,7 +14667,7 @@
         <v>152</v>
       </c>
       <c r="N20" s="132" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="O20" s="132"/>
       <c r="P20" s="132"/>
@@ -14682,7 +14682,7 @@
     </row>
     <row r="21" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A21" s="132" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="B21" s="132"/>
       <c r="C21" s="132"/>
@@ -14690,7 +14690,7 @@
       <c r="E21" s="132"/>
       <c r="F21" s="132"/>
       <c r="N21" s="132" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="O21" s="132"/>
       <c r="P21" s="132"/>
@@ -14700,7 +14700,7 @@
     </row>
     <row r="22" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A22" s="132" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="B22" s="132"/>
       <c r="C22" s="132"/>
@@ -14713,7 +14713,7 @@
         <v>152</v>
       </c>
       <c r="N22" s="132" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="O22" s="132"/>
       <c r="P22" s="132"/>
@@ -14728,7 +14728,7 @@
     </row>
     <row r="23" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A23" s="132" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="B23" s="132"/>
       <c r="C23" s="132"/>
@@ -14741,7 +14741,7 @@
         <v>152</v>
       </c>
       <c r="N23" s="132" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="O23" s="132"/>
       <c r="P23" s="132"/>
@@ -14756,7 +14756,7 @@
     </row>
     <row r="24" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A24" s="132" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="B24" s="132"/>
       <c r="C24" s="132"/>
@@ -14769,7 +14769,7 @@
         <v>152</v>
       </c>
       <c r="N24" s="132" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="O24" s="132"/>
       <c r="P24" s="132"/>
@@ -14784,7 +14784,7 @@
     </row>
     <row r="25" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A25" s="132" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="B25" s="132"/>
       <c r="C25" s="132"/>
@@ -14797,7 +14797,7 @@
         <v>152</v>
       </c>
       <c r="N25" s="132" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="O25" s="132"/>
       <c r="P25" s="132"/>
@@ -14812,7 +14812,7 @@
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A26" s="132" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="B26" s="132"/>
       <c r="C26" s="132"/>
@@ -14825,7 +14825,7 @@
         <v>152</v>
       </c>
       <c r="N26" s="132" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="O26" s="132"/>
       <c r="P26" s="132"/>
@@ -14840,7 +14840,7 @@
     </row>
     <row r="27" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A27" s="132" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="B27" s="132"/>
       <c r="C27" s="132"/>
@@ -14853,7 +14853,7 @@
         <v>152</v>
       </c>
       <c r="N27" s="132" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="O27" s="132"/>
       <c r="P27" s="132"/>
@@ -14868,7 +14868,7 @@
     </row>
     <row r="28" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A28" s="132" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="B28" s="132"/>
       <c r="C28" s="132"/>
@@ -14881,7 +14881,7 @@
         <v>152</v>
       </c>
       <c r="N28" s="132" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="O28" s="132"/>
       <c r="P28" s="132"/>
@@ -14896,7 +14896,7 @@
     </row>
     <row r="30" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A30" s="132" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="B30" s="132"/>
       <c r="C30" s="132"/>
@@ -14909,7 +14909,7 @@
         <v>152</v>
       </c>
       <c r="N30" s="132" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="O30" s="132"/>
       <c r="P30" s="132"/>
@@ -14924,7 +14924,7 @@
     </row>
     <row r="31" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A31" s="132" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="B31" s="132"/>
       <c r="C31" s="132"/>
@@ -14937,7 +14937,7 @@
         <v>152</v>
       </c>
       <c r="H31" s="132" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="I31" s="132"/>
       <c r="J31" s="132"/>
@@ -14947,10 +14947,10 @@
         <v>10000</v>
       </c>
       <c r="M31" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="N31" s="132" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="O31" s="132"/>
       <c r="P31" s="132"/>
@@ -14965,7 +14965,7 @@
     </row>
     <row r="32" spans="1:19" x14ac:dyDescent="0.3">
       <c r="H32" s="132" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="I32" s="132"/>
       <c r="J32" s="132"/>
@@ -14977,7 +14977,7 @@
     </row>
     <row r="33" spans="1:19" x14ac:dyDescent="0.3">
       <c r="H33" s="132" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="I33" s="132"/>
       <c r="J33" s="132"/>
@@ -14988,13 +14988,13 @@
     </row>
     <row r="34" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A34" s="132" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="B34" s="132"/>
       <c r="C34" s="132"/>
       <c r="D34" s="132"/>
       <c r="H34" s="132" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="I34" s="132"/>
       <c r="J34" s="132"/>
@@ -15003,7 +15003,7 @@
         <v>1</v>
       </c>
       <c r="N34" s="132" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="O34" s="132"/>
       <c r="P34" s="132"/>
@@ -15011,14 +15011,14 @@
     </row>
     <row r="35" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A35" s="132" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="B35" s="132"/>
       <c r="C35" s="132"/>
       <c r="D35" s="132"/>
       <c r="E35" s="132"/>
       <c r="H35" s="132" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="I35" s="132"/>
       <c r="J35" s="132"/>
@@ -15027,7 +15027,7 @@
         <v>0</v>
       </c>
       <c r="N35" s="132" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="O35" s="132"/>
       <c r="P35" s="132"/>
@@ -15036,7 +15036,7 @@
     </row>
     <row r="36" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A36" s="132" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="B36" s="132"/>
       <c r="C36" s="132"/>
@@ -15049,7 +15049,7 @@
         <v>152</v>
       </c>
       <c r="H36" s="132" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="I36" s="132"/>
       <c r="J36" s="132"/>
@@ -15058,7 +15058,7 @@
         <v>1</v>
       </c>
       <c r="N36" s="132" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="O36" s="132"/>
       <c r="P36" s="132"/>
@@ -15073,7 +15073,7 @@
     </row>
     <row r="37" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A37" s="132" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="B37" s="132"/>
       <c r="C37" s="132"/>
@@ -15086,7 +15086,7 @@
         <v>152</v>
       </c>
       <c r="H37" s="132" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="I37" s="132"/>
       <c r="J37" s="132"/>
@@ -15095,7 +15095,7 @@
         <v>1.6</v>
       </c>
       <c r="N37" s="132" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="O37" s="132"/>
       <c r="P37" s="132"/>
@@ -15110,7 +15110,7 @@
     </row>
     <row r="38" spans="1:19" x14ac:dyDescent="0.3">
       <c r="H38" s="132" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="I38" s="132"/>
       <c r="J38" s="132"/>
@@ -15121,14 +15121,14 @@
     </row>
     <row r="39" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A39" s="132" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="B39" s="132"/>
       <c r="C39" s="132"/>
       <c r="D39" s="132"/>
       <c r="E39" s="132"/>
       <c r="H39" s="132" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="I39" s="132"/>
       <c r="J39" s="132"/>
@@ -15137,7 +15137,7 @@
         <v>1</v>
       </c>
       <c r="N39" s="132" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="O39" s="132"/>
       <c r="P39" s="132"/>
@@ -15146,7 +15146,7 @@
     </row>
     <row r="40" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A40" s="132" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="B40" s="132"/>
       <c r="C40" s="132"/>
@@ -15159,7 +15159,7 @@
         <v>152</v>
       </c>
       <c r="H40" s="132" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="I40" s="132"/>
       <c r="J40" s="132"/>
@@ -15169,7 +15169,7 @@
         <v>22</v>
       </c>
       <c r="N40" s="132" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="O40" s="132"/>
       <c r="P40" s="132"/>
@@ -15184,7 +15184,7 @@
     </row>
     <row r="41" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A41" s="132" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="B41" s="132"/>
       <c r="C41" s="132"/>
@@ -15195,7 +15195,7 @@
       </c>
       <c r="F41" s="132"/>
       <c r="H41" s="132" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="I41" s="132"/>
       <c r="J41" s="132"/>
@@ -15205,7 +15205,7 @@
         <v>3</v>
       </c>
       <c r="N41" s="132" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="O41" s="132"/>
       <c r="P41" s="132"/>
@@ -15218,7 +15218,7 @@
     </row>
     <row r="42" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A42" s="132" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="B42" s="132"/>
       <c r="C42" s="132"/>
@@ -15229,7 +15229,7 @@
       </c>
       <c r="F42" s="132"/>
       <c r="H42" s="132" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="I42" s="132"/>
       <c r="J42" s="132"/>
@@ -15238,7 +15238,7 @@
         <v>0.63</v>
       </c>
       <c r="N42" s="132" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="O42" s="132"/>
       <c r="P42" s="132"/>
@@ -15251,7 +15251,7 @@
     </row>
     <row r="44" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A44" s="132" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="B44" s="132"/>
       <c r="C44" s="132"/>
@@ -15264,7 +15264,7 @@
         <v>16</v>
       </c>
       <c r="N44" s="132" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="O44" s="132"/>
       <c r="P44" s="132"/>
@@ -15279,7 +15279,7 @@
     </row>
     <row r="45" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A45" s="132" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="B45" s="132"/>
       <c r="C45" s="132"/>
@@ -15292,7 +15292,7 @@
         <v>317</v>
       </c>
       <c r="N45" s="132" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="O45" s="132"/>
       <c r="P45" s="132"/>
@@ -15307,7 +15307,7 @@
     </row>
     <row r="46" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A46" s="132" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="B46" s="132"/>
       <c r="C46" s="132"/>
@@ -15320,7 +15320,7 @@
         <v>57</v>
       </c>
       <c r="N46" s="132" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="O46" s="132"/>
       <c r="P46" s="132"/>
@@ -15335,7 +15335,7 @@
     </row>
     <row r="48" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A48" s="132" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="B48" s="132"/>
       <c r="C48" s="132"/>
@@ -15347,7 +15347,7 @@
         <v>57</v>
       </c>
       <c r="N48" s="132" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="O48" s="132"/>
       <c r="P48" s="132"/>
@@ -15361,7 +15361,7 @@
     </row>
     <row r="49" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A49" s="132" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="B49" s="132"/>
       <c r="C49" s="132"/>
@@ -15374,7 +15374,7 @@
         <v>152</v>
       </c>
       <c r="N49" s="132" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="O49" s="132"/>
       <c r="P49" s="132"/>
@@ -15395,19 +15395,19 @@
         <v>327</v>
       </c>
       <c r="C51" t="s">
+        <v>416</v>
+      </c>
+      <c r="D51" t="s">
+        <v>422</v>
+      </c>
+      <c r="E51" t="s">
         <v>417</v>
       </c>
-      <c r="D51" t="s">
-        <v>423</v>
-      </c>
-      <c r="E51" t="s">
+      <c r="F51" t="s">
+        <v>419</v>
+      </c>
+      <c r="G51" t="s">
         <v>418</v>
-      </c>
-      <c r="F51" t="s">
-        <v>420</v>
-      </c>
-      <c r="G51" t="s">
-        <v>419</v>
       </c>
       <c r="N51" t="s">
         <v>193</v>
@@ -15416,19 +15416,19 @@
         <v>327</v>
       </c>
       <c r="P51" t="s">
+        <v>416</v>
+      </c>
+      <c r="Q51" t="s">
+        <v>422</v>
+      </c>
+      <c r="R51" t="s">
         <v>417</v>
       </c>
-      <c r="Q51" t="s">
-        <v>423</v>
-      </c>
-      <c r="R51" t="s">
+      <c r="S51" t="s">
+        <v>419</v>
+      </c>
+      <c r="T51" t="s">
         <v>418</v>
-      </c>
-      <c r="S51" t="s">
-        <v>420</v>
-      </c>
-      <c r="T51" t="s">
-        <v>419</v>
       </c>
     </row>
     <row r="52" spans="1:20" x14ac:dyDescent="0.3">
@@ -15479,7 +15479,7 @@
     </row>
     <row r="54" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A54" s="132" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="B54" s="132"/>
       <c r="C54" s="132"/>
@@ -15492,7 +15492,7 @@
         <v>57</v>
       </c>
       <c r="N54" s="132" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="O54" s="132"/>
       <c r="P54" s="132"/>
@@ -15518,7 +15518,7 @@
       </c>
       <c r="F55" s="132"/>
       <c r="G55" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="N55" s="132" t="s">
         <v>137</v>
@@ -15532,12 +15532,12 @@
       </c>
       <c r="S55" s="132"/>
       <c r="T55" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="56" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A56" s="132" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="B56" s="132"/>
       <c r="C56" s="132"/>
@@ -15548,7 +15548,7 @@
       </c>
       <c r="F56" s="132"/>
       <c r="N56" s="132" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="O56" s="132"/>
       <c r="P56" s="132"/>
@@ -15910,7 +15910,7 @@
     </row>
     <row r="17" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A17" s="132" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="B17" s="132"/>
       <c r="C17" s="132"/>
@@ -15920,12 +15920,12 @@
         <v>0.39332459432785055</v>
       </c>
       <c r="F17" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
     </row>
     <row r="18" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A18" s="132" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="B18" s="132"/>
       <c r="C18" s="132"/>
@@ -15940,7 +15940,7 @@
     </row>
     <row r="19" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A19" s="132" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="B19" s="132"/>
       <c r="C19" s="132"/>
@@ -15955,7 +15955,7 @@
     </row>
     <row r="20" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A20" s="132" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="B20" s="132"/>
       <c r="C20" s="132"/>
@@ -15995,7 +15995,7 @@
     </row>
     <row r="22" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A22" s="132" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="B22" s="132"/>
       <c r="C22" s="132"/>
@@ -16016,7 +16016,7 @@
     </row>
     <row r="23" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A23" s="132" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="B23" s="132"/>
       <c r="C23" s="132"/>
@@ -16031,7 +16031,7 @@
     </row>
     <row r="24" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A24" s="132" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="B24" s="132"/>
       <c r="C24" s="132"/>
@@ -16123,10 +16123,10 @@
         <v>320</v>
       </c>
       <c r="F31" s="101" t="s">
+        <v>455</v>
+      </c>
+      <c r="G31" t="s">
         <v>456</v>
-      </c>
-      <c r="G31" t="s">
-        <v>457</v>
       </c>
     </row>
     <row r="32" spans="1:23" x14ac:dyDescent="0.3">

</xml_diff>